<commit_message>
Brand assets, hero visual, and section polish across homepage
- New hero brand image + ServiceVisual/BenefitMark components
- Refreshed favicons, logo, OG image and generator script
- Contact/CTA/Services/Showcase section refinements
- Update salon-demo and salon-retro submodule pointers
- Import cowork agent instructions (AGENTS.md, .agents/)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Appinara_Prospekti_a_Outreach.xlsx
+++ b/Appinara_Prospekti_a_Outreach.xlsx
@@ -650,7 +650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N248"/>
+  <dimension ref="A1:N311"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="10" min="1" max="1"/>
@@ -4204,10 +4204,14 @@
       </c>
       <c r="K54" s="10" t="inlineStr">
         <is>
-          <t>Draft pripravený</t>
-        </is>
-      </c>
-      <c r="L54" s="10" t="inlineStr"/>
+          <t>Odoslané</t>
+        </is>
+      </c>
+      <c r="L54" s="10" t="inlineStr">
+        <is>
+          <t>08.07.2026</t>
+        </is>
+      </c>
       <c r="M54" s="10" t="inlineStr">
         <is>
           <t>Pilates štúdio BA centrum, blízko Vivo. Skupinové lekcie max 10 ľudí, individuálne, rehab, prenatal. Od 06/2025 aj masáže. Rezervácie cez vlastný systém pilatesmy.sk/res/. Hook: chýba FAQ pre prvonávštevníka.</t>
@@ -4332,10 +4336,14 @@
       </c>
       <c r="K56" s="10" t="inlineStr">
         <is>
-          <t>Draft pripravený</t>
-        </is>
-      </c>
-      <c r="L56" s="10" t="inlineStr"/>
+          <t>Odoslané</t>
+        </is>
+      </c>
+      <c r="L56" s="10" t="inlineStr">
+        <is>
+          <t>08.07.2026</t>
+        </is>
+      </c>
       <c r="M56" s="10" t="inlineStr">
         <is>
           <t>Beckovská 29 BA. Zakladateľka = fyzioterapeutka + certifikovaná pilates instruktorka od 2010. Apparatus equipment z USA (Reformer Trapeze, Studio Reformer, Exo Chair). Hook: 2 typy klientov (akútny vs preventívny) potrebujú triáž pred lekciou.</t>
@@ -4658,10 +4666,14 @@
       </c>
       <c r="K61" s="10" t="inlineStr">
         <is>
-          <t>Draft pripravený</t>
-        </is>
-      </c>
-      <c r="L61" s="10" t="inlineStr"/>
+          <t>Odoslané</t>
+        </is>
+      </c>
+      <c r="L61" s="10" t="inlineStr">
+        <is>
+          <t>08.07.2026</t>
+        </is>
+      </c>
       <c r="M61" s="10" t="inlineStr">
         <is>
           <t>Košice. Po-Pi 10-14, So-Ne na objednávku. Hlavná služba: denné menu + takeaway. Objednávky telefonicky do 11:00 (+421 55 642 5081). Hook: ranné okno 9:30-11:00 zahltené telefonátmi 'aké máte dnes menu'.</t>
@@ -4720,10 +4732,14 @@
       </c>
       <c r="K62" s="10" t="inlineStr">
         <is>
-          <t>Draft pripravený</t>
-        </is>
-      </c>
-      <c r="L62" s="10" t="inlineStr"/>
+          <t>Odoslané</t>
+        </is>
+      </c>
+      <c r="L62" s="10" t="inlineStr">
+        <is>
+          <t>08.07.2026</t>
+        </is>
+      </c>
       <c r="M62" s="10" t="inlineStr">
         <is>
           <t>Žilina, pri vodnej priehrade. Po-Ne 10-22. Rodinný biznis De Riggo. Rezervácie cez priamy telefón (Robert / Alena). Doručovanie cez bistro.sk. Hook: cez sezónu non-stop telefón na rodinné mobily.</t>
@@ -16439,6 +16455,3928 @@
         </is>
       </c>
       <c r="N248" s="21" t="inlineStr"/>
+    </row>
+    <row r="249">
+      <c r="A249" s="13" t="n">
+        <v>288</v>
+      </c>
+      <c r="B249" s="13" t="inlineStr">
+        <is>
+          <t>E-shop</t>
+        </is>
+      </c>
+      <c r="C249" s="14" t="inlineStr">
+        <is>
+          <t>BBZOO</t>
+        </is>
+      </c>
+      <c r="D249" s="14" t="inlineStr">
+        <is>
+          <t>https://www.bbzoo.sk</t>
+        </is>
+      </c>
+      <c r="E249" s="14" t="inlineStr">
+        <is>
+          <t>eshop@bbzoo.sk</t>
+        </is>
+      </c>
+      <c r="F249" s="13" t="inlineStr">
+        <is>
+          <t>0915 754 855</t>
+        </is>
+      </c>
+      <c r="G249" s="13" t="inlineStr">
+        <is>
+          <t>Trnava</t>
+        </is>
+      </c>
+      <c r="H249" s="14" t="inlineStr">
+        <is>
+          <t>AI poradca odpovie na výber krmiva a vybavenia 24/7 (aj po 12:00) a čerpá z ich Poradne</t>
+        </is>
+      </c>
+      <c r="I249" s="14" t="inlineStr">
+        <is>
+          <t>Rozšírená podpora / knowledge z blogu</t>
+        </is>
+      </c>
+      <c r="J249" s="13" t="inlineStr">
+        <is>
+          <t>Vysoká</t>
+        </is>
+      </c>
+      <c r="K249" s="13" t="inlineStr">
+        <is>
+          <t>Draft pripravený</t>
+        </is>
+      </c>
+      <c r="L249" s="13" t="n"/>
+      <c r="M249" s="14" t="inlineStr">
+        <is>
+          <t>E-shop bez kamennej predajne, obrovský katalóg (psy, mačky, vtáky, akvaristika, teraristika, hospodárske zvieratá). Tel. podpora len 9-12h, e-mail nonstop. Silná Poradňa/blog (domáci zverolekár). Hook: 24/7 poradca čerpajúci z Poradne.</t>
+        </is>
+      </c>
+      <c r="N249" s="21" t="n"/>
+    </row>
+    <row r="250">
+      <c r="A250" s="13" t="n">
+        <v>289</v>
+      </c>
+      <c r="B250" s="13" t="inlineStr">
+        <is>
+          <t>E-shop</t>
+        </is>
+      </c>
+      <c r="C250" s="14" t="inlineStr">
+        <is>
+          <t>JAPITEX</t>
+        </is>
+      </c>
+      <c r="D250" s="14" t="inlineStr">
+        <is>
+          <t>https://www.japitex.sk</t>
+        </is>
+      </c>
+      <c r="E250" s="14" t="inlineStr">
+        <is>
+          <t>eshop@japitex.sk</t>
+        </is>
+      </c>
+      <c r="F250" s="13" t="inlineStr">
+        <is>
+          <t>0944 353 060</t>
+        </is>
+      </c>
+      <c r="G250" s="13" t="inlineStr">
+        <is>
+          <t>Slovensko (export SK/CZ/HU/HR)</t>
+        </is>
+      </c>
+      <c r="H250" s="14" t="inlineStr">
+        <is>
+          <t>AI veľkostný poradca pre dojčenské/detské oblečenie, multijazyčný pre CZ/HU/HR trhy</t>
+        </is>
+      </c>
+      <c r="I250" s="14" t="inlineStr">
+        <is>
+          <t>Veľkostný poradca + multilingual</t>
+        </is>
+      </c>
+      <c r="J250" s="13" t="inlineStr">
+        <is>
+          <t>Vysoká</t>
+        </is>
+      </c>
+      <c r="K250" s="13" t="inlineStr">
+        <is>
+          <t>Draft pripravený</t>
+        </is>
+      </c>
+      <c r="L250" s="13" t="n"/>
+      <c r="M250" s="14" t="inlineStr">
+        <is>
+          <t>Výrobca a predajca dojčenského/detského oblečenia (0-14 r.) + ženy/muži. Weby SK/CZ/HU/HR/EN. Majú tabuľku veľkostí. Hook: rodičia tápu vo veľkostiach 0-1 vs 2-6 -&gt; AI poradca znižuje vratky.</t>
+        </is>
+      </c>
+      <c r="N250" s="21" t="n"/>
+    </row>
+    <row r="251">
+      <c r="A251" s="13" t="n">
+        <v>290</v>
+      </c>
+      <c r="B251" s="13" t="inlineStr">
+        <is>
+          <t>E-shop</t>
+        </is>
+      </c>
+      <c r="C251" s="14" t="inlineStr">
+        <is>
+          <t>AZ Dom a Záhrada</t>
+        </is>
+      </c>
+      <c r="D251" s="14" t="inlineStr">
+        <is>
+          <t>https://www.az-domazahrada.sk</t>
+        </is>
+      </c>
+      <c r="E251" s="14" t="inlineStr">
+        <is>
+          <t>azdomazahrada@gmail.com</t>
+        </is>
+      </c>
+      <c r="F251" s="13" t="inlineStr">
+        <is>
+          <t>0948 071 337 / 0915 625 310</t>
+        </is>
+      </c>
+      <c r="G251" s="13" t="inlineStr">
+        <is>
+          <t>Slovensko</t>
+        </is>
+      </c>
+      <c r="H251" s="14" t="inlineStr">
+        <is>
+          <t>AI poradca odporučí konkrétny postrek/hnojivo podľa problému alebo tvarovku podľa rozmeru</t>
+        </is>
+      </c>
+      <c r="I251" s="14" t="inlineStr">
+        <is>
+          <t>Poradca v technickom sortimente</t>
+        </is>
+      </c>
+      <c r="J251" s="13" t="inlineStr">
+        <is>
+          <t>Stredná</t>
+        </is>
+      </c>
+      <c r="K251" s="13" t="inlineStr">
+        <is>
+          <t>Odoslané</t>
+        </is>
+      </c>
+      <c r="L251" s="13" t="inlineStr">
+        <is>
+          <t>09.07.2026</t>
+        </is>
+      </c>
+      <c r="M251" s="14" t="inlineStr">
+        <is>
+          <t>E-shop záhrada + dom + voda/plyn/kúrenie. Odborný sortiment (fungicídy, insekticídy, KG/HT kanalizácia, PEX, batérie po sériách). Dve rôzne kontaktné čísla (záhrada vs voda). Hook: 'aký postrek na akú chorobu'.</t>
+        </is>
+      </c>
+      <c r="N251" s="21" t="n"/>
+    </row>
+    <row r="252">
+      <c r="A252" s="13" t="n">
+        <v>291</v>
+      </c>
+      <c r="B252" s="13" t="inlineStr">
+        <is>
+          <t>E-shop</t>
+        </is>
+      </c>
+      <c r="C252" s="14" t="inlineStr">
+        <is>
+          <t>Pražiarnička</t>
+        </is>
+      </c>
+      <c r="D252" s="14" t="inlineStr">
+        <is>
+          <t>https://praziarnicka.sk</t>
+        </is>
+      </c>
+      <c r="E252" s="14" t="inlineStr">
+        <is>
+          <t>info@praziarnicka.sk</t>
+        </is>
+      </c>
+      <c r="F252" s="13" t="inlineStr">
+        <is>
+          <t>+421 917 502 991</t>
+        </is>
+      </c>
+      <c r="G252" s="13" t="inlineStr">
+        <is>
+          <t>Trenčín</t>
+        </is>
+      </c>
+      <c r="H252" s="14" t="inlineStr">
+        <is>
+          <t>AI poradca odporučí kávu podľa chuti + zachytí B2B dopyt na dodávky do firiem</t>
+        </is>
+      </c>
+      <c r="I252" s="14" t="inlineStr">
+        <is>
+          <t>Chuťový poradca + B2B lead</t>
+        </is>
+      </c>
+      <c r="J252" s="13" t="inlineStr">
+        <is>
+          <t>Stredná</t>
+        </is>
+      </c>
+      <c r="K252" s="13" t="inlineStr">
+        <is>
+          <t>Odoslané</t>
+        </is>
+      </c>
+      <c r="L252" s="13" t="inlineStr">
+        <is>
+          <t>09.07.2026</t>
+        </is>
+      </c>
+      <c r="M252" s="14" t="inlineStr">
+        <is>
+          <t>Pražiareň + kaviareň (Štúrovo nám. Trenčín) + e-shop + sekcia Pre firmy. Vlastné blendy (Paganini, Puccini), arabica. Hook: výber zrna na e-shope + B2B dopyty na pravidelné dodávky.</t>
+        </is>
+      </c>
+      <c r="N252" s="21" t="n"/>
+    </row>
+    <row r="253">
+      <c r="A253" s="13" t="n">
+        <v>292</v>
+      </c>
+      <c r="B253" s="13" t="inlineStr">
+        <is>
+          <t>E-shop</t>
+        </is>
+      </c>
+      <c r="C253" s="14" t="inlineStr">
+        <is>
+          <t>Anipet</t>
+        </is>
+      </c>
+      <c r="D253" s="14" t="inlineStr">
+        <is>
+          <t>https://www.anipet.sk</t>
+        </is>
+      </c>
+      <c r="E253" s="14" t="inlineStr">
+        <is>
+          <t>obchod@anipet.sk</t>
+        </is>
+      </c>
+      <c r="F253" s="13" t="inlineStr">
+        <is>
+          <t>+421 903 890 359</t>
+        </is>
+      </c>
+      <c r="G253" s="13" t="inlineStr">
+        <is>
+          <t>Bratislava / Trnava / Nitra</t>
+        </is>
+      </c>
+      <c r="H253" s="14" t="inlineStr">
+        <is>
+          <t>AI poradca pre výber krmiva + smerovanie na dostupnosť a najbližšiu predajňu (omnichannel)</t>
+        </is>
+      </c>
+      <c r="I253" s="14" t="inlineStr">
+        <is>
+          <t>Omnichannel poradca + knowledge z blogu</t>
+        </is>
+      </c>
+      <c r="J253" s="13" t="inlineStr">
+        <is>
+          <t>Stredná</t>
+        </is>
+      </c>
+      <c r="K253" s="13" t="inlineStr">
+        <is>
+          <t>Odoslané</t>
+        </is>
+      </c>
+      <c r="L253" s="13" t="inlineStr">
+        <is>
+          <t>09.07.2026</t>
+        </is>
+      </c>
+      <c r="M253" s="14" t="inlineStr">
+        <is>
+          <t>Chovateľské potreby od 2004, e-shop + predajne (DNV Bratislava, Trnava, Nitra Centro + Ferenitka). Široký sortiment značiek, bonusový program, blog 'Rady a tipy'. Hook: dostupnosť medzi predajňami + výber krmiva.</t>
+        </is>
+      </c>
+      <c r="N253" s="21" t="n"/>
+    </row>
+    <row r="254">
+      <c r="A254" s="13" t="n">
+        <v>293</v>
+      </c>
+      <c r="B254" s="13" t="inlineStr">
+        <is>
+          <t>Zdravotníctvo</t>
+        </is>
+      </c>
+      <c r="C254" s="14" t="inlineStr">
+        <is>
+          <t>FYMED</t>
+        </is>
+      </c>
+      <c r="D254" s="14" t="inlineStr">
+        <is>
+          <t>https://www.fymed.sk</t>
+        </is>
+      </c>
+      <c r="E254" s="14" t="inlineStr">
+        <is>
+          <t>rehabilitacia@fymed.sk</t>
+        </is>
+      </c>
+      <c r="F254" s="13" t="inlineStr">
+        <is>
+          <t>0948 572 703</t>
+        </is>
+      </c>
+      <c r="G254" s="13" t="inlineStr">
+        <is>
+          <t>Nitra / Vráble</t>
+        </is>
+      </c>
+      <c r="H254" s="14" t="inlineStr">
+        <is>
+          <t>AI navádza pacienta na správnu pobočku a deň, rieši časté otázky a žiadosť o termín 24/7</t>
+        </is>
+      </c>
+      <c r="I254" s="14" t="inlineStr">
+        <is>
+          <t>Booking + navigácia medzi pobočkami</t>
+        </is>
+      </c>
+      <c r="J254" s="13" t="inlineStr">
+        <is>
+          <t>Vysoká</t>
+        </is>
+      </c>
+      <c r="K254" s="13" t="inlineStr">
+        <is>
+          <t>Odoslané</t>
+        </is>
+      </c>
+      <c r="L254" s="13" t="inlineStr">
+        <is>
+          <t>09.07.2026</t>
+        </is>
+      </c>
+      <c r="M254" s="14" t="inlineStr">
+        <is>
+          <t>Rehabilitačné ambulancie FBLR Nitra + Vráble. Rôzne ordinačné dni na pobočkách (Nitra Po/St/Št, Vráble Ut/St/Pi), 2 tel. čísla, do 15:30. Poisťovne Dôvera/VšZP/Union. Majú Najčastejšie otázky. Hook: zámena dňa/pobočky pri tel. objednaní.</t>
+        </is>
+      </c>
+      <c r="N254" s="21" t="n"/>
+    </row>
+    <row r="255">
+      <c r="A255" s="13" t="n">
+        <v>294</v>
+      </c>
+      <c r="B255" s="13" t="inlineStr">
+        <is>
+          <t>Zdravotníctvo</t>
+        </is>
+      </c>
+      <c r="C255" s="14" t="inlineStr">
+        <is>
+          <t>Dermatop</t>
+        </is>
+      </c>
+      <c r="D255" s="14" t="inlineStr">
+        <is>
+          <t>https://www.dermatop.sk</t>
+        </is>
+      </c>
+      <c r="E255" s="14" t="inlineStr">
+        <is>
+          <t>dermatop@dermatop.sk</t>
+        </is>
+      </c>
+      <c r="F255" s="13" t="inlineStr">
+        <is>
+          <t>0948 616 000</t>
+        </is>
+      </c>
+      <c r="G255" s="13" t="inlineStr">
+        <is>
+          <t>Trenčín / Partizánske / Dubnica n. Váhom</t>
+        </is>
+      </c>
+      <c r="H255" s="14" t="inlineStr">
+        <is>
+          <t>AI zachytí záujem o zákrok, odpovie na cenu/rekonvalescenciu a pošle žiadosť o termín 24/7</t>
+        </is>
+      </c>
+      <c r="I255" s="14" t="inlineStr">
+        <is>
+          <t>Booking estetiky mimo preťaženého telefónu</t>
+        </is>
+      </c>
+      <c r="J255" s="13" t="inlineStr">
+        <is>
+          <t>Vysoká</t>
+        </is>
+      </c>
+      <c r="K255" s="13" t="inlineStr">
+        <is>
+          <t>Odoslané</t>
+        </is>
+      </c>
+      <c r="L255" s="13" t="inlineStr">
+        <is>
+          <t>09.07.2026</t>
+        </is>
+      </c>
+      <c r="M255" s="14" t="inlineStr">
+        <is>
+          <t>Estetické a laserové centrum, 3 pobočky. Sami na webe prosia o trpezlivosť pri telefonátoch a možnosť nechať SMS. Online objednanie len pre kožnú ambulanciu (topdoktor), estetika cez telefón. Hook: preťažený telefón na estetiku.</t>
+        </is>
+      </c>
+      <c r="N255" s="21" t="n"/>
+    </row>
+    <row r="256">
+      <c r="A256" s="13" t="n">
+        <v>295</v>
+      </c>
+      <c r="B256" s="13" t="inlineStr">
+        <is>
+          <t>Zdravotníctvo</t>
+        </is>
+      </c>
+      <c r="C256" s="14" t="inlineStr">
+        <is>
+          <t>zubko (MUDr. Peter Ladányi)</t>
+        </is>
+      </c>
+      <c r="D256" s="14" t="inlineStr">
+        <is>
+          <t>https://www.zubko.sk</t>
+        </is>
+      </c>
+      <c r="E256" s="14" t="inlineStr"/>
+      <c r="F256" s="13" t="inlineStr">
+        <is>
+          <t>055/643 07 63</t>
+        </is>
+      </c>
+      <c r="G256" s="13" t="inlineStr">
+        <is>
+          <t>Košice</t>
+        </is>
+      </c>
+      <c r="H256" s="14" t="inlineStr">
+        <is>
+          <t>AI FAQ + booking pre solo ordináciu (majú vlastnú FAQ stránku)</t>
+        </is>
+      </c>
+      <c r="I256" s="14" t="inlineStr">
+        <is>
+          <t>FAQ/booking bot</t>
+        </is>
+      </c>
+      <c r="J256" s="13" t="inlineStr">
+        <is>
+          <t>Nízka</t>
+        </is>
+      </c>
+      <c r="K256" s="13" t="inlineStr">
+        <is>
+          <t>Email chýba</t>
+        </is>
+      </c>
+      <c r="L256" s="13" t="n"/>
+      <c r="M256" s="14" t="inlineStr">
+        <is>
+          <t>Solo zubná ordinácia (bielenie, dentálna hygiena, implantológia), Trieda SNP 407/61 Košice. Web na Hostinger builderi, majú FAQ stránku. Objednanie len telefonicky. Na webe NIE je e-mail -&gt; draft nevytvorený, treba dohľadať kontaktný e-mail.</t>
+        </is>
+      </c>
+      <c r="N256" s="21" t="n"/>
+    </row>
+    <row r="257">
+      <c r="A257" s="13" t="n">
+        <v>296</v>
+      </c>
+      <c r="B257" s="13" t="inlineStr">
+        <is>
+          <t>Zdravotníctvo</t>
+        </is>
+      </c>
+      <c r="C257" s="14" t="inlineStr">
+        <is>
+          <t>Klinika Zdravia – kožná ambulancia Žilina</t>
+        </is>
+      </c>
+      <c r="D257" s="14" t="inlineStr">
+        <is>
+          <t>https://www.dermatologicka-klinika.sk</t>
+        </is>
+      </c>
+      <c r="E257" s="14" t="inlineStr"/>
+      <c r="F257" s="13" t="inlineStr">
+        <is>
+          <t>+421 950 526 846</t>
+        </is>
+      </c>
+      <c r="G257" s="13" t="inlineStr">
+        <is>
+          <t>Žilina (OC Tambor)</t>
+        </is>
+      </c>
+      <c r="H257" s="14" t="inlineStr">
+        <is>
+          <t>AI triáž kožných problémov + objednanie na presný čas 24/7</t>
+        </is>
+      </c>
+      <c r="I257" s="14" t="inlineStr">
+        <is>
+          <t>Triáž + booking</t>
+        </is>
+      </c>
+      <c r="J257" s="13" t="inlineStr">
+        <is>
+          <t>Stredná</t>
+        </is>
+      </c>
+      <c r="K257" s="13" t="inlineStr">
+        <is>
+          <t>Email chýba</t>
+        </is>
+      </c>
+      <c r="L257" s="13" t="n"/>
+      <c r="M257" s="14" t="inlineStr">
+        <is>
+          <t>Súkromná kožná ambulancia (3 ambulancie, vlastná operačná sála, lasery ADVATx, PicoLO). Objednávajú na presný čas, dlhá ordinačná doba. E-mail na webe je zahmlený (JS obfuskácia) -&gt; treba dohľadať pred draftom.</t>
+        </is>
+      </c>
+      <c r="N257" s="21" t="n"/>
+    </row>
+    <row r="258">
+      <c r="A258" s="13" t="n">
+        <v>297</v>
+      </c>
+      <c r="B258" s="13" t="inlineStr">
+        <is>
+          <t>Fitness/Wellness</t>
+        </is>
+      </c>
+      <c r="C258" s="14" t="inlineStr">
+        <is>
+          <t>Fit Sport Training</t>
+        </is>
+      </c>
+      <c r="D258" s="14" t="inlineStr">
+        <is>
+          <t>https://fst.sk</t>
+        </is>
+      </c>
+      <c r="E258" s="14" t="inlineStr">
+        <is>
+          <t>info@fst.sk</t>
+        </is>
+      </c>
+      <c r="F258" s="13" t="inlineStr">
+        <is>
+          <t>+421 904 55 24 87</t>
+        </is>
+      </c>
+      <c r="G258" s="13" t="inlineStr">
+        <is>
+          <t>Zvolen / Banská Bystrica</t>
+        </is>
+      </c>
+      <c r="H258" s="14" t="inlineStr">
+        <is>
+          <t>AI zachytí nováčika pri 'bezplatnej konzultácii', odporučí program a rezervuje termín 24/7</t>
+        </is>
+      </c>
+      <c r="I258" s="14" t="inlineStr">
+        <is>
+          <t>Lead z bezplatnej konzultácie</t>
+        </is>
+      </c>
+      <c r="J258" s="13" t="inlineStr">
+        <is>
+          <t>Vysoká</t>
+        </is>
+      </c>
+      <c r="K258" s="13" t="inlineStr">
+        <is>
+          <t>Odoslané</t>
+        </is>
+      </c>
+      <c r="L258" s="13" t="inlineStr">
+        <is>
+          <t>09.07.2026</t>
+        </is>
+      </c>
+      <c r="M258" s="14" t="inlineStr">
+        <is>
+          <t>Netradičné tréningové centrum (nie klasické fitko), Zvolen + BB. Ponuka: individuálne, skupinové, Fit kids, cvičenie pre tehotné, Fit health (fyzio/masáže). Na webe formulár 'Bezplatná konzultácia'. Hook: zachytenie leadu skôr, než opadne motivácia.</t>
+        </is>
+      </c>
+      <c r="N258" s="21" t="n"/>
+    </row>
+    <row r="259">
+      <c r="A259" s="13" t="n">
+        <v>298</v>
+      </c>
+      <c r="B259" s="13" t="inlineStr">
+        <is>
+          <t>Fitness/Wellness</t>
+        </is>
+      </c>
+      <c r="C259" s="14" t="inlineStr">
+        <is>
+          <t>MM Fitness</t>
+        </is>
+      </c>
+      <c r="D259" s="14" t="inlineStr">
+        <is>
+          <t>https://mmfitness.sk</t>
+        </is>
+      </c>
+      <c r="E259" s="14" t="inlineStr"/>
+      <c r="F259" s="13" t="inlineStr">
+        <is>
+          <t>048/4145145</t>
+        </is>
+      </c>
+      <c r="G259" s="13" t="inlineStr">
+        <is>
+          <t>Banská Bystrica</t>
+        </is>
+      </c>
+      <c r="H259" s="14" t="inlineStr">
+        <is>
+          <t>AI odpovie na cenník/MultiSport/otváracie hodiny + rezervuje InBody meranie a PT</t>
+        </is>
+      </c>
+      <c r="I259" s="14" t="inlineStr">
+        <is>
+          <t>FAQ + booking merania/PT</t>
+        </is>
+      </c>
+      <c r="J259" s="13" t="inlineStr">
+        <is>
+          <t>Nízka</t>
+        </is>
+      </c>
+      <c r="K259" s="13" t="inlineStr">
+        <is>
+          <t>Email chýba</t>
+        </is>
+      </c>
+      <c r="L259" s="13" t="n"/>
+      <c r="M259" s="14" t="inlineStr">
+        <is>
+          <t>Posilňovňa 550 m², 80 strojov, Hammer Strength official training center, InBody 370S meranie tela, MultiSport/Benefit Plus. Medený Hámor, BB. Na webe len telefón + kontaktný formulár, NIE je e-mail -&gt; draft nevytvorený.</t>
+        </is>
+      </c>
+      <c r="N259" s="21" t="n"/>
+    </row>
+    <row r="260">
+      <c r="A260" s="13" t="n">
+        <v>299</v>
+      </c>
+      <c r="B260" s="13" t="inlineStr">
+        <is>
+          <t>Gastro</t>
+        </is>
+      </c>
+      <c r="C260" s="14" t="inlineStr">
+        <is>
+          <t>Koliba Neresnica</t>
+        </is>
+      </c>
+      <c r="D260" s="14" t="inlineStr">
+        <is>
+          <t>https://kolibaneresnica.sk</t>
+        </is>
+      </c>
+      <c r="E260" s="14" t="inlineStr">
+        <is>
+          <t>kolibaneresnica@gmail.com</t>
+        </is>
+      </c>
+      <c r="F260" s="13" t="inlineStr">
+        <is>
+          <t>045/532 34 06</t>
+        </is>
+      </c>
+      <c r="G260" s="13" t="inlineStr">
+        <is>
+          <t>Zvolen</t>
+        </is>
+      </c>
+      <c r="H260" s="14" t="inlineStr">
+        <is>
+          <t>AI prijme rezerváciu stola/altánku + rieši voľné miesta v kempingu, spojí dva kanály</t>
+        </is>
+      </c>
+      <c r="I260" s="14" t="inlineStr">
+        <is>
+          <t>Rezervačný bot pre kolibu + kemping</t>
+        </is>
+      </c>
+      <c r="J260" s="13" t="inlineStr">
+        <is>
+          <t>Stredná</t>
+        </is>
+      </c>
+      <c r="K260" s="13" t="inlineStr">
+        <is>
+          <t>Draft pripravený</t>
+        </is>
+      </c>
+      <c r="L260" s="13" t="n"/>
+      <c r="M260" s="14" t="inlineStr">
+        <is>
+          <t>Slovenská kuchyňa (bryndzové halušky), letný zastrešený altánok, popri kolibe kemping s ubytovaním. Rezervácie telefonicky, koliba a kemping majú samostatné čísla. Hook: hosť potrebuje 2 hovory (stôl + prespanie).</t>
+        </is>
+      </c>
+      <c r="N260" s="21" t="n"/>
+    </row>
+    <row r="261">
+      <c r="A261" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="B261" s="13" t="inlineStr">
+        <is>
+          <t>Gastro</t>
+        </is>
+      </c>
+      <c r="C261" s="14" t="inlineStr">
+        <is>
+          <t>Trnavský dvor</t>
+        </is>
+      </c>
+      <c r="D261" s="14" t="inlineStr">
+        <is>
+          <t>https://www.trnavskydvor.sk</t>
+        </is>
+      </c>
+      <c r="E261" s="14" t="inlineStr"/>
+      <c r="F261" s="13" t="inlineStr">
+        <is>
+          <t>0901 71 71 61</t>
+        </is>
+      </c>
+      <c r="G261" s="13" t="inlineStr">
+        <is>
+          <t>Trnava</t>
+        </is>
+      </c>
+      <c r="H261" s="14" t="inlineStr">
+        <is>
+          <t>AI prijíma objednávky denného menu/rozvozu + dopyty na eventy (svadby, gril na býka)</t>
+        </is>
+      </c>
+      <c r="I261" s="14" t="inlineStr">
+        <is>
+          <t>Objednávky + eventy</t>
+        </is>
+      </c>
+      <c r="J261" s="13" t="inlineStr">
+        <is>
+          <t>Stredná</t>
+        </is>
+      </c>
+      <c r="K261" s="13" t="inlineStr">
+        <is>
+          <t>Email chýba</t>
+        </is>
+      </c>
+      <c r="L261" s="13" t="n"/>
+      <c r="M261" s="14" t="inlineStr">
+        <is>
+          <t>TOP reštaurácia Trnavy 20 rokov, denné menu s rozvozom (objednávky telefonicky od 8:00), pizza donáška, sála 90 osôb na svadby/firemné akcie, gril na býka, letné akcie so živou kapelou. E-mail na webe skrytý cez JavaScript -&gt; treba dohľadať pred draftom.</t>
+        </is>
+      </c>
+      <c r="N261" s="21" t="n"/>
+    </row>
+    <row r="262">
+      <c r="A262" s="13" t="n">
+        <v>301</v>
+      </c>
+      <c r="B262" s="13" t="inlineStr">
+        <is>
+          <t>Gastro</t>
+        </is>
+      </c>
+      <c r="C262" s="14" t="inlineStr">
+        <is>
+          <t>Restaurant Veža</t>
+        </is>
+      </c>
+      <c r="D262" s="14" t="inlineStr">
+        <is>
+          <t>https://www.restaurantveza.sk</t>
+        </is>
+      </c>
+      <c r="E262" s="14" t="inlineStr"/>
+      <c r="F262" s="13" t="inlineStr"/>
+      <c r="G262" s="13" t="inlineStr">
+        <is>
+          <t>Liptovský Mikuláš</t>
+        </is>
+      </c>
+      <c r="H262" s="14" t="inlineStr">
+        <is>
+          <t>AI rezervácia stola + info o dennom menu a eventoch (oslavy, rodinné posedenia)</t>
+        </is>
+      </c>
+      <c r="I262" s="14" t="inlineStr">
+        <is>
+          <t>Rezervačný bot</t>
+        </is>
+      </c>
+      <c r="J262" s="13" t="inlineStr">
+        <is>
+          <t>Nízka</t>
+        </is>
+      </c>
+      <c r="K262" s="13" t="inlineStr">
+        <is>
+          <t>Email chýba</t>
+        </is>
+      </c>
+      <c r="L262" s="13" t="n"/>
+      <c r="M262" s="14" t="inlineStr">
+        <is>
+          <t>Reštaurácia (Kamenné pole 4558/14, Liptovský Mikuláš), denné menu, oslavy a eventy na mieru. Otvorené len 11:00-16:00 (So do 14:00). Na webe pole E-mail prázdne -&gt; draft nevytvorený, treba dohľadať kontakt.</t>
+        </is>
+      </c>
+      <c r="N262" s="21" t="n"/>
+    </row>
+    <row r="263">
+      <c r="A263" s="13" t="n">
+        <v>302</v>
+      </c>
+      <c r="B263" s="13" t="inlineStr">
+        <is>
+          <t>Hotel/Penzión</t>
+        </is>
+      </c>
+      <c r="C263" s="14" t="inlineStr">
+        <is>
+          <t>Penzión Panorama (Nízke Tatry)</t>
+        </is>
+      </c>
+      <c r="D263" s="14" t="inlineStr">
+        <is>
+          <t>https://www.panoramapenzion.sk</t>
+        </is>
+      </c>
+      <c r="E263" s="14" t="inlineStr">
+        <is>
+          <t>info@panoramapenzion.sk</t>
+        </is>
+      </c>
+      <c r="F263" s="13" t="inlineStr"/>
+      <c r="G263" s="13" t="inlineStr">
+        <is>
+          <t>Nízke Tatry</t>
+        </is>
+      </c>
+      <c r="H263" s="14" t="inlineStr">
+        <is>
+          <t>AI concierge + booking automation, multijazyčný pre zahraničných hostí</t>
+        </is>
+      </c>
+      <c r="I263" s="14" t="inlineStr">
+        <is>
+          <t>Concierge + booking</t>
+        </is>
+      </c>
+      <c r="J263" s="13" t="inlineStr">
+        <is>
+          <t>Stredná</t>
+        </is>
+      </c>
+      <c r="K263" s="13" t="inlineStr">
+        <is>
+          <t>Treba lepší research</t>
+        </is>
+      </c>
+      <c r="L263" s="13" t="n"/>
+      <c r="M263" s="14" t="inlineStr">
+        <is>
+          <t>Nový penzión v Nízkych Tatrách s vyhrievaným vonkajším bazénom a wellness (podľa listingu). E-mail info@panoramapenzion.sk. Homepage sa nepodarilo načítať (JS/provenance) -&gt; pred draftom treba overiť web a konkrétny hook.</t>
+        </is>
+      </c>
+      <c r="N263" s="21" t="n"/>
+    </row>
+    <row r="264">
+      <c r="A264" s="13" t="n">
+        <v>303</v>
+      </c>
+      <c r="B264" s="13" t="inlineStr">
+        <is>
+          <t>Reality</t>
+        </is>
+      </c>
+      <c r="C264" s="14" t="inlineStr">
+        <is>
+          <t>FOK realitná kancelária</t>
+        </is>
+      </c>
+      <c r="D264" s="14" t="inlineStr">
+        <is>
+          <t>https://fok.sk</t>
+        </is>
+      </c>
+      <c r="E264" s="14" t="inlineStr">
+        <is>
+          <t>fok@fok.sk</t>
+        </is>
+      </c>
+      <c r="F264" s="13" t="inlineStr">
+        <is>
+          <t>0905 276 401</t>
+        </is>
+      </c>
+      <c r="G264" s="13" t="inlineStr">
+        <is>
+          <t>Prešov</t>
+        </is>
+      </c>
+      <c r="H264" s="14" t="inlineStr">
+        <is>
+          <t>AI predkvalifikuje záujemcov (rozpočet, lokalita, typ) a odovzdá maklérovi pripravený lead</t>
+        </is>
+      </c>
+      <c r="I264" s="14" t="inlineStr">
+        <is>
+          <t>Kvalifikácia leadov pred obhliadkou</t>
+        </is>
+      </c>
+      <c r="J264" s="13" t="inlineStr">
+        <is>
+          <t>Vysoká</t>
+        </is>
+      </c>
+      <c r="K264" s="13" t="inlineStr">
+        <is>
+          <t>Odoslané</t>
+        </is>
+      </c>
+      <c r="L264" s="13" t="inlineStr">
+        <is>
+          <t>09.07.2026</t>
+        </is>
+      </c>
+      <c r="M264" s="14" t="inlineStr">
+        <is>
+          <t>Najdlhšie existujúca RK v Prešove (od 1992, 25+ rokov), Jarková 59. Video-obhliadka zdarma, kompletný právny servis, Poradňa/blog. Referencie zdôrazňujú rýchlosť (nájomca do pár dní). Hook: prvotné otázky k inzerátom zaberajú maklérom čas.</t>
+        </is>
+      </c>
+      <c r="N264" s="21" t="n"/>
+    </row>
+    <row r="265">
+      <c r="A265" s="13" t="n">
+        <v>304</v>
+      </c>
+      <c r="B265" s="13" t="inlineStr">
+        <is>
+          <t>Reality</t>
+        </is>
+      </c>
+      <c r="C265" s="14" t="inlineStr">
+        <is>
+          <t>Nitrianska realitná kancelária</t>
+        </is>
+      </c>
+      <c r="D265" s="14" t="inlineStr">
+        <is>
+          <t>https://nitrianskereality.com</t>
+        </is>
+      </c>
+      <c r="E265" s="14" t="inlineStr">
+        <is>
+          <t>reality@nitrianskereality.com</t>
+        </is>
+      </c>
+      <c r="F265" s="13" t="inlineStr">
+        <is>
+          <t>0910 747 333</t>
+        </is>
+      </c>
+      <c r="G265" s="13" t="inlineStr">
+        <is>
+          <t>Nitra</t>
+        </is>
+      </c>
+      <c r="H265" s="14" t="inlineStr">
+        <is>
+          <t>AI osloví majiteľa hneď po dopyte z formulára, doplní údaje a odovzdá pripravený lead</t>
+        </is>
+      </c>
+      <c r="I265" s="14" t="inlineStr">
+        <is>
+          <t>Rýchla reakcia na formulár na ohodnotenie</t>
+        </is>
+      </c>
+      <c r="J265" s="13" t="inlineStr">
+        <is>
+          <t>Vysoká</t>
+        </is>
+      </c>
+      <c r="K265" s="13" t="inlineStr">
+        <is>
+          <t>Odoslané</t>
+        </is>
+      </c>
+      <c r="L265" s="13" t="inlineStr">
+        <is>
+          <t>09.07.2026</t>
+        </is>
+      </c>
+      <c r="M265" s="14" t="inlineStr">
+        <is>
+          <t>RK Nitra (Farská 9), tím maklérov, home staging, foto/dron, cenové stanovisko do 48h. Na webe formulár 'Chcete poznať hodnotu svojej nehnuteľnosti?'. Hook: ticho medzi vyplnením formulára a odpoveďou -&gt; časť majiteľov vychladne.</t>
+        </is>
+      </c>
+      <c r="N265" s="21" t="n"/>
+    </row>
+    <row r="266">
+      <c r="A266" s="13" t="n">
+        <v>305</v>
+      </c>
+      <c r="B266" s="13" t="inlineStr">
+        <is>
+          <t>E-shop</t>
+        </is>
+      </c>
+      <c r="C266" s="14" t="inlineStr">
+        <is>
+          <t>Graano</t>
+        </is>
+      </c>
+      <c r="D266" s="14" t="inlineStr">
+        <is>
+          <t>https://www.graano.sk</t>
+        </is>
+      </c>
+      <c r="E266" s="14" t="inlineStr">
+        <is>
+          <t>graanocoffee@gmail.com</t>
+        </is>
+      </c>
+      <c r="F266" s="13" t="inlineStr">
+        <is>
+          <t>+421 949 849 468</t>
+        </is>
+      </c>
+      <c r="G266" s="13" t="inlineStr">
+        <is>
+          <t>Bratislava / Orava (Tvrdošín)</t>
+        </is>
+      </c>
+      <c r="H266" s="14" t="inlineStr">
+        <is>
+          <t>Sprievodca na webe, ktorý podľa zámeru (predplatné / espresso / darček na svadbu) odporučí konkrétnu zrnkovku a balenie</t>
+        </is>
+      </c>
+      <c r="I266" s="14" t="inlineStr">
+        <is>
+          <t>Guide sekcia 3 – jedna observácia (3 typy zákazníkov) → jeden nápad (AI product picker)</t>
+        </is>
+      </c>
+      <c r="J266" s="13" t="inlineStr">
+        <is>
+          <t>Vysoká</t>
+        </is>
+      </c>
+      <c r="K266" s="13" t="inlineStr">
+        <is>
+          <t>Draft pripravený</t>
+        </is>
+      </c>
+      <c r="L266" s="13" t="inlineStr"/>
+      <c r="M266" s="14" t="inlineStr">
+        <is>
+          <t>Remeselná pražiareň, praží na Orave, odberné miesto Tvrdošín. Ponúka predplatné, kávu na svadby aj balíčky pre firmy. Hravé názvy pôvodov (Dobrodružný Jaguár, Bystrý Medveď). Bez chatbota.</t>
+        </is>
+      </c>
+      <c r="N266" s="21" t="inlineStr"/>
+    </row>
+    <row r="267">
+      <c r="A267" s="13" t="n">
+        <v>306</v>
+      </c>
+      <c r="B267" s="13" t="inlineStr">
+        <is>
+          <t>E-shop</t>
+        </is>
+      </c>
+      <c r="C267" s="14" t="inlineStr">
+        <is>
+          <t>Wilfred</t>
+        </is>
+      </c>
+      <c r="D267" s="14" t="inlineStr">
+        <is>
+          <t>https://www.wilfred.sk</t>
+        </is>
+      </c>
+      <c r="E267" s="14" t="inlineStr">
+        <is>
+          <t>david@wilfred.sk</t>
+        </is>
+      </c>
+      <c r="F267" s="13" t="inlineStr">
+        <is>
+          <t>+421 908 205 403</t>
+        </is>
+      </c>
+      <c r="G267" s="13" t="inlineStr">
+        <is>
+          <t>Slažany</t>
+        </is>
+      </c>
+      <c r="H267" s="14" t="inlineStr">
+        <is>
+          <t>AI sprievodca, ktorý podľa nálady/príležitosti odporučí čaj z ponuky (vrátane Aphroditea, darčekové balíky)</t>
+        </is>
+      </c>
+      <c r="I267" s="14" t="inlineStr">
+        <is>
+          <t>Guide sekcia 3 – zrkadlenie existujúcej 'Mám chuť...' navigácie</t>
+        </is>
+      </c>
+      <c r="J267" s="13" t="inlineStr">
+        <is>
+          <t>Vysoká</t>
+        </is>
+      </c>
+      <c r="K267" s="13" t="inlineStr">
+        <is>
+          <t>Draft pripravený</t>
+        </is>
+      </c>
+      <c r="L267" s="13" t="inlineStr"/>
+      <c r="M267" s="14" t="inlineStr">
+        <is>
+          <t>Rodinná čajová dielňa, ručne balené čaje, držiteľ 5 hviezd Great Taste Awards. Web triedi čaje podľa nálady (Mám chuť byť plný energie/uvoľnený/gurmán). Firemné darčeky a poukazy. Bez chatbota.</t>
+        </is>
+      </c>
+      <c r="N267" s="21" t="inlineStr"/>
+    </row>
+    <row r="268">
+      <c r="A268" s="13" t="n">
+        <v>307</v>
+      </c>
+      <c r="B268" s="13" t="inlineStr">
+        <is>
+          <t>E-shop</t>
+        </is>
+      </c>
+      <c r="C268" s="14" t="inlineStr">
+        <is>
+          <t>Ready After</t>
+        </is>
+      </c>
+      <c r="D268" s="14" t="inlineStr">
+        <is>
+          <t>https://www.readyafter.sk</t>
+        </is>
+      </c>
+      <c r="E268" s="14" t="inlineStr">
+        <is>
+          <t>kava@readyafter.sk</t>
+        </is>
+      </c>
+      <c r="F268" s="13" t="inlineStr">
+        <is>
+          <t>+421 948 137 204</t>
+        </is>
+      </c>
+      <c r="G268" s="13" t="inlineStr">
+        <is>
+          <t>Slovensko</t>
+        </is>
+      </c>
+      <c r="H268" s="14" t="inlineStr">
+        <is>
+          <t>AI sprievodca výberom kávy podľa spôsobu prípravy, chuti a kávovaru; obsluha aj B2B dopytov</t>
+        </is>
+      </c>
+      <c r="I268" s="14" t="inlineStr">
+        <is>
+          <t>Guide sekcia 3 – naviazané na ich kategorizáciu podľa kyslosti + stránku 'Ako vybrať kávu'</t>
+        </is>
+      </c>
+      <c r="J268" s="13" t="inlineStr">
+        <is>
+          <t>Stredná</t>
+        </is>
+      </c>
+      <c r="K268" s="13" t="inlineStr">
+        <is>
+          <t>Draft pripravený</t>
+        </is>
+      </c>
+      <c r="L268" s="13" t="inlineStr"/>
+      <c r="M268" s="14" t="inlineStr">
+        <is>
+          <t>Pražiareň 20+ rokov, zrno priamo z vietnamskej farmy. Kávu triedi podľa krajiny, kyslosti a chuťového profilu. B2B: kaviareň, kancelária, branding. Bez chatbota.</t>
+        </is>
+      </c>
+      <c r="N268" s="21" t="inlineStr"/>
+    </row>
+    <row r="269">
+      <c r="A269" s="13" t="n">
+        <v>308</v>
+      </c>
+      <c r="B269" s="13" t="inlineStr">
+        <is>
+          <t>E-shop</t>
+        </is>
+      </c>
+      <c r="C269" s="14" t="inlineStr">
+        <is>
+          <t>Froggywear</t>
+        </is>
+      </c>
+      <c r="D269" s="14" t="inlineStr">
+        <is>
+          <t>https://froggywear.sk</t>
+        </is>
+      </c>
+      <c r="E269" s="14" t="inlineStr">
+        <is>
+          <t>obchod@froggywear.sk</t>
+        </is>
+      </c>
+      <c r="F269" s="13" t="inlineStr">
+        <is>
+          <t>+421 950 357 443</t>
+        </is>
+      </c>
+      <c r="G269" s="13" t="inlineStr">
+        <is>
+          <t>Šamorín</t>
+        </is>
+      </c>
+      <c r="H269" s="14" t="inlineStr">
+        <is>
+          <t>AI poradca veľkosti/hrúbky merina podľa veku dieťaťa, aktivity a obdobia; odpovede na časté otázky (cena vs. syntetika)</t>
+        </is>
+      </c>
+      <c r="I269" s="14" t="inlineStr">
+        <is>
+          <t>Guide sekcia 3 – zložitosť výberu (veľkosť 56-164 × aktivita × obdobie) → jeden AI poradca</t>
+        </is>
+      </c>
+      <c r="J269" s="13" t="inlineStr">
+        <is>
+          <t>Vysoká</t>
+        </is>
+      </c>
+      <c r="K269" s="13" t="inlineStr">
+        <is>
+          <t>Draft pripravený</t>
+        </is>
+      </c>
+      <c r="L269" s="13" t="inlineStr"/>
+      <c r="M269" s="14" t="inlineStr">
+        <is>
+          <t>Navrhnuté a šité na SK (dielňa Šamorín), merino pre celú rodinu. Ponuka triedená podľa aktivity (turistika, cyklo, nosenie detí, kancelária), 'rastúce' kúsky pre bábätká. Manuálny Messenger/WhatsApp, žiadny AI bot.</t>
+        </is>
+      </c>
+      <c r="N269" s="21" t="inlineStr"/>
+    </row>
+    <row r="270">
+      <c r="A270" s="13" t="n">
+        <v>309</v>
+      </c>
+      <c r="B270" s="13" t="inlineStr">
+        <is>
+          <t>E-shop</t>
+        </is>
+      </c>
+      <c r="C270" s="14" t="inlineStr">
+        <is>
+          <t>Sviečočka</t>
+        </is>
+      </c>
+      <c r="D270" s="14" t="inlineStr">
+        <is>
+          <t>https://sviecocka.sk</t>
+        </is>
+      </c>
+      <c r="E270" s="14" t="inlineStr">
+        <is>
+          <t>info@sviecocka.sk</t>
+        </is>
+      </c>
+      <c r="F270" s="13" t="inlineStr">
+        <is>
+          <t>+421 904 886 162</t>
+        </is>
+      </c>
+      <c r="G270" s="13" t="inlineStr">
+        <is>
+          <t>Bratislava</t>
+        </is>
+      </c>
+      <c r="H270" s="14" t="inlineStr">
+        <is>
+          <t>AI sprievodca darčekom – podľa obdarovaného a príležitosti odporučí sviečku aj s vhodným odkazom</t>
+        </is>
+      </c>
+      <c r="I270" s="14" t="inlineStr">
+        <is>
+          <t>Guide sekcia 3 – naviazané na ich členenie podľa príležitosti</t>
+        </is>
+      </c>
+      <c r="J270" s="13" t="inlineStr">
+        <is>
+          <t>Stredná</t>
+        </is>
+      </c>
+      <c r="K270" s="13" t="inlineStr">
+        <is>
+          <t>Draft pripravený</t>
+        </is>
+      </c>
+      <c r="L270" s="13" t="inlineStr"/>
+      <c r="M270" s="14" t="inlineStr">
+        <is>
+          <t>Ručne vyrábané sójové sviečky s osobným odkazom, výroba na SK. Katalóg členený podľa príležitosti (Deň matiek, svadba, pre starých rodičov, koniec šk. roka) a sezóny. Moderný web (Next.js), vernostný program. Bez chatbota.</t>
+        </is>
+      </c>
+      <c r="N270" s="21" t="inlineStr"/>
+    </row>
+    <row r="271">
+      <c r="A271" s="13" t="n">
+        <v>310</v>
+      </c>
+      <c r="B271" s="13" t="inlineStr">
+        <is>
+          <t>Zdravotníctvo</t>
+        </is>
+      </c>
+      <c r="C271" s="14" t="inlineStr">
+        <is>
+          <t>Dentika</t>
+        </is>
+      </c>
+      <c r="D271" s="14" t="inlineStr">
+        <is>
+          <t>https://www.dentika.sk</t>
+        </is>
+      </c>
+      <c r="E271" s="14" t="inlineStr">
+        <is>
+          <t>dentikanr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F271" s="13" t="inlineStr">
+        <is>
+          <t>+421 911 05 12 12</t>
+        </is>
+      </c>
+      <c r="G271" s="13" t="inlineStr">
+        <is>
+          <t>Nitra</t>
+        </is>
+      </c>
+      <c r="H271" s="14" t="inlineStr">
+        <is>
+          <t>AI asistent 24/7 na bežné otázky + zápis žiadostí o termín mimo ordinačných hodín; ranný zoznam pre kliniku</t>
+        </is>
+      </c>
+      <c r="I271" s="14" t="inlineStr">
+        <is>
+          <t>Guide sekcia 4 – zubár, alternatíva k telefónu na rezerváciu</t>
+        </is>
+      </c>
+      <c r="J271" s="13" t="inlineStr">
+        <is>
+          <t>Vysoká</t>
+        </is>
+      </c>
+      <c r="K271" s="13" t="inlineStr">
+        <is>
+          <t>FU1 odoslané</t>
+        </is>
+      </c>
+      <c r="L271" s="13" t="inlineStr">
+        <is>
+          <t>14.07.2026</t>
+        </is>
+      </c>
+      <c r="M271" s="14" t="inlineStr">
+        <is>
+          <t>Mladá klinika MDDr. Ján Korbela (Coboriho 11), RTG/CBCT a mikroskop, prijíma deti. Objednávanie len cez formulár/telefón, pohotovosť 'po telefonickom dohovore', víkend zatvorené. Bez chatbota. | Oprava 10.07.2026: mail reálne odoslaný 08.07.2026, Excel mal zastaraný stav.</t>
+        </is>
+      </c>
+      <c r="N271" s="21" t="inlineStr">
+        <is>
+          <t>08.07.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="13" t="n">
+        <v>311</v>
+      </c>
+      <c r="B272" s="13" t="inlineStr">
+        <is>
+          <t>Zdravotníctvo</t>
+        </is>
+      </c>
+      <c r="C272" s="14" t="inlineStr">
+        <is>
+          <t>Zubné centrum Nitra (Dr. Stanko)</t>
+        </is>
+      </c>
+      <c r="D272" s="14" t="inlineStr">
+        <is>
+          <t>https://www.drstanko.sk</t>
+        </is>
+      </c>
+      <c r="E272" s="14" t="inlineStr">
+        <is>
+          <t>drstanko@drstanko.sk</t>
+        </is>
+      </c>
+      <c r="F272" s="13" t="inlineStr">
+        <is>
+          <t>0948 577 715</t>
+        </is>
+      </c>
+      <c r="G272" s="13" t="inlineStr">
+        <is>
+          <t>Nitra</t>
+        </is>
+      </c>
+      <c r="H272" s="14" t="inlineStr">
+        <is>
+          <t>AI asistent na webe, ktorý okamžite odpovie na otázky (estetika, implantáty, hygiena) a zapíše dopyt na termín</t>
+        </is>
+      </c>
+      <c r="I272" s="14" t="inlineStr">
+        <is>
+          <t>Guide sekcia 4 – zrýchlenie existujúcej sekcie 'Spýtajte sa'</t>
+        </is>
+      </c>
+      <c r="J272" s="13" t="inlineStr">
+        <is>
+          <t>Stredná</t>
+        </is>
+      </c>
+      <c r="K272" s="13" t="inlineStr">
+        <is>
+          <t>Draft pripravený</t>
+        </is>
+      </c>
+      <c r="L272" s="13" t="inlineStr"/>
+      <c r="M272" s="14" t="inlineStr">
+        <is>
+          <t>MUDr. Michal Stanko (Štúrova 103, Mlynárce), aj mklinik.eu. Estetika, implantáty, protetika, hygiena. Web má sekciu 'Spýtajte sa', kde pacienti posielajú otázky. Starší web (2018). Bez chatbota.</t>
+        </is>
+      </c>
+      <c r="N272" s="21" t="inlineStr"/>
+    </row>
+    <row r="273">
+      <c r="A273" s="13" t="n">
+        <v>312</v>
+      </c>
+      <c r="B273" s="13" t="inlineStr">
+        <is>
+          <t>Zdravotníctvo</t>
+        </is>
+      </c>
+      <c r="C273" s="14" t="inlineStr">
+        <is>
+          <t>Fyzioactive</t>
+        </is>
+      </c>
+      <c r="D273" s="14" t="inlineStr">
+        <is>
+          <t>https://fyzioactive.sk</t>
+        </is>
+      </c>
+      <c r="E273" s="14" t="inlineStr">
+        <is>
+          <t>fyzioactive@fyzioactive.sk</t>
+        </is>
+      </c>
+      <c r="F273" s="13" t="inlineStr">
+        <is>
+          <t>+421 948 074 788</t>
+        </is>
+      </c>
+      <c r="G273" s="13" t="inlineStr">
+        <is>
+          <t>Trenčín-Kubrá</t>
+        </is>
+      </c>
+      <c r="H273" s="14" t="inlineStr">
+        <is>
+          <t>AI asistent, ktorý podľa ťažkostí nasmeruje pacienta k vhodnej terapii a k online rezervácii; odpovede pred príchodom</t>
+        </is>
+      </c>
+      <c r="I273" s="14" t="inlineStr">
+        <is>
+          <t>Guide sekcia 4 – naviazané na ich sekciu 'Ako vám môžeme pomôcť' (25+ terapií)</t>
+        </is>
+      </c>
+      <c r="J273" s="13" t="inlineStr">
+        <is>
+          <t>Stredná</t>
+        </is>
+      </c>
+      <c r="K273" s="13" t="inlineStr">
+        <is>
+          <t>Draft pripravený</t>
+        </is>
+      </c>
+      <c r="L273" s="13" t="inlineStr"/>
+      <c r="M273" s="14" t="inlineStr">
+        <is>
+          <t>Ambulancia MUDr. Linda Králiková, 25+ terapií (laser, rázová vlna, SIS magnet), hodnotenie 5,0 / 29+ recenzií. Už má online rezerváciu a FAQ, ale žiadneho AI asistenta na výber terapie.</t>
+        </is>
+      </c>
+      <c r="N273" s="21" t="inlineStr"/>
+    </row>
+    <row r="274">
+      <c r="A274" s="13" t="n">
+        <v>313</v>
+      </c>
+      <c r="B274" s="13" t="inlineStr">
+        <is>
+          <t>Zdravotníctvo</t>
+        </is>
+      </c>
+      <c r="C274" s="14" t="inlineStr">
+        <is>
+          <t>Fyzio-Care</t>
+        </is>
+      </c>
+      <c r="D274" s="14" t="inlineStr">
+        <is>
+          <t>https://www.fyzio-care.sk</t>
+        </is>
+      </c>
+      <c r="E274" s="14" t="inlineStr">
+        <is>
+          <t>info@fyzioterapeuttrencin.sk</t>
+        </is>
+      </c>
+      <c r="F274" s="13" t="inlineStr">
+        <is>
+          <t>0902 219 866</t>
+        </is>
+      </c>
+      <c r="G274" s="13" t="inlineStr">
+        <is>
+          <t>Trenčín</t>
+        </is>
+      </c>
+      <c r="H274" s="14" t="inlineStr">
+        <is>
+          <t>AI asistent, ktorý odpovie na otázky (metódy, na čo pomáhajú, ako sa objednať) a zapíše žiadosť o termín – odbremenenie majiteľa</t>
+        </is>
+      </c>
+      <c r="I274" s="14" t="inlineStr">
+        <is>
+          <t>Guide sekcia 4 – naviazané na jeho vlastné tvrdenie '85 hodín týždenne / 24-7'</t>
+        </is>
+      </c>
+      <c r="J274" s="13" t="inlineStr">
+        <is>
+          <t>Stredná</t>
+        </is>
+      </c>
+      <c r="K274" s="13" t="inlineStr">
+        <is>
+          <t>Draft pripravený</t>
+        </is>
+      </c>
+      <c r="L274" s="13" t="inlineStr"/>
+      <c r="M274" s="14" t="inlineStr">
+        <is>
+          <t>Solo fyzioterapeut PhDr. Šimon Ilkyw (Horný Šianec), zameraný na športovcov, veľký zoznam metód (Graston, McKenzie, dry needling, DNS). Na webe uvádza dostupnosť takmer 24/7 a ~85 h/týždeň. Starší web (2019), kontakt len cez formulár. Bez chatbota.</t>
+        </is>
+      </c>
+      <c r="N274" s="21" t="inlineStr"/>
+    </row>
+    <row r="275">
+      <c r="A275" s="13" t="n">
+        <v>314</v>
+      </c>
+      <c r="B275" s="13" t="inlineStr">
+        <is>
+          <t>Fitness/Wellness</t>
+        </is>
+      </c>
+      <c r="C275" s="14" t="inlineStr">
+        <is>
+          <t>Body Movement</t>
+        </is>
+      </c>
+      <c r="D275" s="14" t="inlineStr">
+        <is>
+          <t>https://www.bodymovement.sk</t>
+        </is>
+      </c>
+      <c r="E275" s="14" t="inlineStr">
+        <is>
+          <t>info@bodymovement.sk</t>
+        </is>
+      </c>
+      <c r="F275" s="13" t="inlineStr">
+        <is>
+          <t>+421 905 060 900</t>
+        </is>
+      </c>
+      <c r="G275" s="13" t="inlineStr">
+        <is>
+          <t>Košice</t>
+        </is>
+      </c>
+      <c r="H275" s="14" t="inlineStr">
+        <is>
+          <t>AI asistent, ktorý podľa cieľa (spevnenie, regenerácia, tehotenstvo) odporučí službu a nasmeruje na online rezerváciu</t>
+        </is>
+      </c>
+      <c r="I275" s="14" t="inlineStr">
+        <is>
+          <t>Guide sekcia 3 – naviazané na ich manuálne CTA 'Chcem sa poradiť'</t>
+        </is>
+      </c>
+      <c r="J275" s="13" t="inlineStr">
+        <is>
+          <t>Stredná</t>
+        </is>
+      </c>
+      <c r="K275" s="13" t="inlineStr">
+        <is>
+          <t>Draft pripravený</t>
+        </is>
+      </c>
+      <c r="L275" s="13" t="inlineStr"/>
+      <c r="M275" s="14" t="inlineStr">
+        <is>
+          <t>Štúdio v Košiciach: Reformer, Pilates, Yoga, GYROTONIC, Barre, cvičenie pre tehotné + masáže (thajské, maderoterapia, bankovanie). Web má mailto 'Chcem sa poradiť' pre výber služby. Online rezervácia áno, chatbot nie.</t>
+        </is>
+      </c>
+      <c r="N275" s="21" t="inlineStr"/>
+    </row>
+    <row r="276">
+      <c r="A276" s="13" t="n">
+        <v>315</v>
+      </c>
+      <c r="B276" s="13" t="inlineStr">
+        <is>
+          <t>Fitness/Wellness</t>
+        </is>
+      </c>
+      <c r="C276" s="14" t="inlineStr">
+        <is>
+          <t>Formery Studio</t>
+        </is>
+      </c>
+      <c r="D276" s="14" t="inlineStr">
+        <is>
+          <t>https://www.formery.studio</t>
+        </is>
+      </c>
+      <c r="E276" s="14" t="inlineStr">
+        <is>
+          <t>hello@formery.studio</t>
+        </is>
+      </c>
+      <c r="F276" s="13" t="inlineStr">
+        <is>
+          <t>+421 910 409 410</t>
+        </is>
+      </c>
+      <c r="G276" s="13" t="inlineStr">
+        <is>
+          <t>Košice / Prešov</t>
+        </is>
+      </c>
+      <c r="H276" s="14" t="inlineStr">
+        <is>
+          <t>AI asistent na výber matwork vs. reformer, rezervácia v správnom meste a otázky k eventom – menej odpisovania v DM</t>
+        </is>
+      </c>
+      <c r="I276" s="14" t="inlineStr">
+        <is>
+          <t>Guide sekcia 3 – dve lokality + plný event kalendár</t>
+        </is>
+      </c>
+      <c r="J276" s="13" t="inlineStr">
+        <is>
+          <t>Stredná</t>
+        </is>
+      </c>
+      <c r="K276" s="13" t="inlineStr">
+        <is>
+          <t>Draft pripravený</t>
+        </is>
+      </c>
+      <c r="L276" s="13" t="inlineStr"/>
+      <c r="M276" s="14" t="inlineStr">
+        <is>
+          <t>Reformer &amp; mat pilates v dvoch mestách (Košice, Prešov), app rezervácie, veľa eventov (outdoor pilates, Golf &amp; Pilates Cup, brunch &amp; pilates). Aktívny Instagram/TikTok. Bez AI bota.</t>
+        </is>
+      </c>
+      <c r="N276" s="21" t="inlineStr"/>
+    </row>
+    <row r="277">
+      <c r="A277" s="13" t="n">
+        <v>316</v>
+      </c>
+      <c r="B277" s="13" t="inlineStr">
+        <is>
+          <t>Fitness/Wellness</t>
+        </is>
+      </c>
+      <c r="C277" s="14" t="inlineStr">
+        <is>
+          <t>Pilates Štúdio Košice</t>
+        </is>
+      </c>
+      <c r="D277" s="14" t="inlineStr">
+        <is>
+          <t>https://www.pilatesstudiokosice.sk</t>
+        </is>
+      </c>
+      <c r="E277" s="14" t="inlineStr">
+        <is>
+          <t>katka@pilatesstudiokosice.sk</t>
+        </is>
+      </c>
+      <c r="F277" s="13" t="inlineStr">
+        <is>
+          <t>+421 917 762 305</t>
+        </is>
+      </c>
+      <c r="G277" s="13" t="inlineStr">
+        <is>
+          <t>Košice</t>
+        </is>
+      </c>
+      <c r="H277" s="14" t="inlineStr">
+        <is>
+          <t>AI asistent, ktorý začiatočníkovi poradí level a typ (matwork/reformer) + obslúži záujemcov o inštruktorské kurzy</t>
+        </is>
+      </c>
+      <c r="I277" s="14" t="inlineStr">
+        <is>
+          <t>Guide sekcia 3 – dve odlišné cieľovky (klienti vs. budúci inštruktori)</t>
+        </is>
+      </c>
+      <c r="J277" s="13" t="inlineStr">
+        <is>
+          <t>Stredná</t>
+        </is>
+      </c>
+      <c r="K277" s="13" t="inlineStr">
+        <is>
+          <t>Draft pripravený</t>
+        </is>
+      </c>
+      <c r="L277" s="13" t="inlineStr"/>
+      <c r="M277" s="14" t="inlineStr">
+        <is>
+          <t>STOTT PILATES, jediné Merrithew Host Training Centrum na SK. Skupinové hodiny (reformer/matwork, level 1-3) aj vzdelávanie inštruktorov. Zakladateľka Katarína Schererová. Online rezervácia, bez chatbota.</t>
+        </is>
+      </c>
+      <c r="N277" s="21" t="inlineStr"/>
+    </row>
+    <row r="278">
+      <c r="A278" s="13" t="n">
+        <v>317</v>
+      </c>
+      <c r="B278" s="13" t="inlineStr">
+        <is>
+          <t>Gastro</t>
+        </is>
+      </c>
+      <c r="C278" s="14" t="inlineStr">
+        <is>
+          <t>Retro Restaurant</t>
+        </is>
+      </c>
+      <c r="D278" s="14" t="inlineStr">
+        <is>
+          <t>https://retrorestaurant.sk</t>
+        </is>
+      </c>
+      <c r="E278" s="14" t="inlineStr">
+        <is>
+          <t>retro@retrorestaurant.sk</t>
+        </is>
+      </c>
+      <c r="F278" s="13" t="inlineStr">
+        <is>
+          <t>+421 908 622 192</t>
+        </is>
+      </c>
+      <c r="G278" s="13" t="inlineStr">
+        <is>
+          <t>Trenčín</t>
+        </is>
+      </c>
+      <c r="H278" s="14" t="inlineStr">
+        <is>
+          <t>AI asistent na webe, ktorý prijme rezerváciu stola aj dopyt na oslavu/akciu a pošle lead na e-mail</t>
+        </is>
+      </c>
+      <c r="I278" s="14" t="inlineStr">
+        <is>
+          <t>Guide sekcia 4 – rezervácie/eventy dnes iba cez telefón</t>
+        </is>
+      </c>
+      <c r="J278" s="13" t="inlineStr">
+        <is>
+          <t>Stredná</t>
+        </is>
+      </c>
+      <c r="K278" s="13" t="inlineStr">
+        <is>
+          <t>Draft pripravený</t>
+        </is>
+      </c>
+      <c r="L278" s="13" t="inlineStr"/>
+      <c r="M278" s="14" t="inlineStr">
+        <is>
+          <t>Reštaurácia v historickom centre Trenčína, tradičná SK + medzinárodná kuchyňa, oslavy/svadby/catering, detský kútik. Menu len ako PDF, rezervácia iba cez 3 telefónne čísla. Bez chatbota.</t>
+        </is>
+      </c>
+      <c r="N278" s="21" t="inlineStr"/>
+    </row>
+    <row r="279">
+      <c r="A279" s="13" t="n">
+        <v>318</v>
+      </c>
+      <c r="B279" s="13" t="inlineStr">
+        <is>
+          <t>Gastro</t>
+        </is>
+      </c>
+      <c r="C279" s="14" t="inlineStr">
+        <is>
+          <t>Terra Mate</t>
+        </is>
+      </c>
+      <c r="D279" s="14" t="inlineStr">
+        <is>
+          <t>https://www.terramate.sk</t>
+        </is>
+      </c>
+      <c r="E279" s="14" t="inlineStr">
+        <is>
+          <t>terramate@bevanda.sk</t>
+        </is>
+      </c>
+      <c r="F279" s="13" t="inlineStr">
+        <is>
+          <t>0907 777 897</t>
+        </is>
+      </c>
+      <c r="G279" s="13" t="inlineStr">
+        <is>
+          <t>Trenčín</t>
+        </is>
+      </c>
+      <c r="H279" s="14" t="inlineStr">
+        <is>
+          <t>AI asistent na rezerváciu stola, dopyt na oslavu (94 miest) aj otázky k donáške – odpoveď hosťovi hneď</t>
+        </is>
+      </c>
+      <c r="I279" s="14" t="inlineStr">
+        <is>
+          <t>Guide sekcia 4 – eventy/donáška/rezervácie dnes hlavne cez telefón</t>
+        </is>
+      </c>
+      <c r="J279" s="13" t="inlineStr">
+        <is>
+          <t>Stredná</t>
+        </is>
+      </c>
+      <c r="K279" s="13" t="inlineStr">
+        <is>
+          <t>Draft pripravený</t>
+        </is>
+      </c>
+      <c r="L279" s="13" t="inlineStr"/>
+      <c r="M279" s="14" t="inlineStr">
+        <is>
+          <t>Reštaurácia v OC MAX Trenčín, kapacita 94, eventy, donáška, degustácie vín, dobre spracované denné menu. Rezervácia a dopyty na akcie hlavne telefonicky. Bez chatbota.</t>
+        </is>
+      </c>
+      <c r="N279" s="21" t="inlineStr"/>
+    </row>
+    <row r="280">
+      <c r="A280" s="13" t="n">
+        <v>319</v>
+      </c>
+      <c r="B280" s="13" t="inlineStr">
+        <is>
+          <t>Gastro</t>
+        </is>
+      </c>
+      <c r="C280" s="14" t="inlineStr">
+        <is>
+          <t>Reštaurácia U Janka</t>
+        </is>
+      </c>
+      <c r="D280" s="14" t="inlineStr">
+        <is>
+          <t>https://www.ujanka.sk</t>
+        </is>
+      </c>
+      <c r="E280" s="14" t="inlineStr">
+        <is>
+          <t>janpitonak13@gmail.com</t>
+        </is>
+      </c>
+      <c r="F280" s="13" t="inlineStr">
+        <is>
+          <t>0907 922 101</t>
+        </is>
+      </c>
+      <c r="G280" s="13" t="inlineStr">
+        <is>
+          <t>Poprad</t>
+        </is>
+      </c>
+      <c r="H280" s="14" t="inlineStr">
+        <is>
+          <t>Moderný mobilný web s viditeľným denným menu + automatická odpoveď na FB na otázky typu 'máte dnes obedy?'</t>
+        </is>
+      </c>
+      <c r="I280" s="14" t="inlineStr">
+        <is>
+          <t>Guide sekcia 4 – tradičný biznis so slabým digitálom</t>
+        </is>
+      </c>
+      <c r="J280" s="13" t="inlineStr">
+        <is>
+          <t>Nízka</t>
+        </is>
+      </c>
+      <c r="K280" s="13" t="inlineStr">
+        <is>
+          <t>Draft pripravený</t>
+        </is>
+      </c>
+      <c r="L280" s="13" t="inlineStr"/>
+      <c r="M280" s="14" t="inlineStr">
+        <is>
+          <t>Malá obedová reštaurácia (Nám. sv. Egídia), domáca kuchyňa, PO-PIA 10-16. Denné menu len ako PDF na stiahnutie, web v podobe z r. 2013, prijíma stravné lístky. Slabší fit (nízky rozpočet), ale konkrétny hook.</t>
+        </is>
+      </c>
+      <c r="N280" s="21" t="inlineStr"/>
+    </row>
+    <row r="281">
+      <c r="A281" s="13" t="n">
+        <v>320</v>
+      </c>
+      <c r="B281" s="13" t="inlineStr">
+        <is>
+          <t>Hotel/Penzión</t>
+        </is>
+      </c>
+      <c r="C281" s="14" t="inlineStr">
+        <is>
+          <t>Penzión Jakub</t>
+        </is>
+      </c>
+      <c r="D281" s="14" t="inlineStr">
+        <is>
+          <t>https://www.penzionjakub.sk</t>
+        </is>
+      </c>
+      <c r="E281" s="14" t="inlineStr">
+        <is>
+          <t>paulik@penzionjakub.sk</t>
+        </is>
+      </c>
+      <c r="F281" s="13" t="inlineStr">
+        <is>
+          <t>+421 907 564 450</t>
+        </is>
+      </c>
+      <c r="G281" s="13" t="inlineStr">
+        <is>
+          <t>Poprad</t>
+        </is>
+      </c>
+      <c r="H281" s="14" t="inlineStr">
+        <is>
+          <t>Dotiahnutie webu + AI asistent na otázky (ubytovanie/reštaurácia/oslavy) a rezerváciu stola; nasaditeľné naprieč skupinou</t>
+        </is>
+      </c>
+      <c r="I281" s="14" t="inlineStr">
+        <is>
+          <t>Guide sekcia 1 – konkrétna observácia (nedokončená šablóna 'Lorem ipsum')</t>
+        </is>
+      </c>
+      <c r="J281" s="13" t="inlineStr">
+        <is>
+          <t>Vysoká</t>
+        </is>
+      </c>
+      <c r="K281" s="13" t="inlineStr">
+        <is>
+          <t>Draft pripravený</t>
+        </is>
+      </c>
+      <c r="L281" s="13" t="inlineStr"/>
+      <c r="M281" s="14" t="inlineStr">
+        <is>
+          <t>Penzión + reštaurácia + sauna + oslavy v Poprade, súčasť skupiny (Alžbetka, Villa Casablanca). Sekcia reštaurácie na webe má stále vzorový text 'Lorem ipsum' a jedlá v dolároch. Rezervácia stola len telefónny odkaz. Bez chatbota.</t>
+        </is>
+      </c>
+      <c r="N281" s="21" t="inlineStr"/>
+    </row>
+    <row r="282">
+      <c r="A282" s="13" t="n">
+        <v>321</v>
+      </c>
+      <c r="B282" s="13" t="inlineStr">
+        <is>
+          <t>Hotel/Penzión</t>
+        </is>
+      </c>
+      <c r="C282" s="14" t="inlineStr">
+        <is>
+          <t>Penzión Roháč</t>
+        </is>
+      </c>
+      <c r="D282" s="14" t="inlineStr">
+        <is>
+          <t>http://www.penzion-rohac.sk</t>
+        </is>
+      </c>
+      <c r="E282" s="14" t="inlineStr">
+        <is>
+          <t>info@penzion-rohac.sk</t>
+        </is>
+      </c>
+      <c r="F282" s="13" t="inlineStr">
+        <is>
+          <t>+421 904 238 388</t>
+        </is>
+      </c>
+      <c r="G282" s="13" t="inlineStr">
+        <is>
+          <t>Zuberec (Roháče)</t>
+        </is>
+      </c>
+      <c r="H282" s="14" t="inlineStr">
+        <is>
+          <t>Moderný web s nezáväznou rezerváciou + viacjazyčný AI asistent (voľné termíny, polpenzia, ORAVA PASS)</t>
+        </is>
+      </c>
+      <c r="I282" s="14" t="inlineStr">
+        <is>
+          <t>Guide sekcia 4 – viacjazyční hostia, ale zastaraný web/formulár</t>
+        </is>
+      </c>
+      <c r="J282" s="13" t="inlineStr">
+        <is>
+          <t>Nízka</t>
+        </is>
+      </c>
+      <c r="K282" s="13" t="inlineStr">
+        <is>
+          <t>Draft pripravený</t>
+        </is>
+      </c>
+      <c r="L282" s="13" t="inlineStr"/>
+      <c r="M282" s="14" t="inlineStr">
+        <is>
+          <t>Malý rodinný penzión v Zuberci, web v SK/PL/DE/HU, polpenzia, požičovňa bicyklov, zľavy ORAVA PASS. Web aj kontaktný formulár pôsobia zastaralo (formulár možno nefunkčný). Malý rozpočet, ale konkrétny viacjazyčný hook.</t>
+        </is>
+      </c>
+      <c r="N282" s="21" t="inlineStr"/>
+    </row>
+    <row r="283">
+      <c r="A283" s="13" t="n">
+        <v>322</v>
+      </c>
+      <c r="B283" s="13" t="inlineStr">
+        <is>
+          <t>Hotel/Penzión</t>
+        </is>
+      </c>
+      <c r="C283" s="14" t="inlineStr">
+        <is>
+          <t>Penzión Pribiskô</t>
+        </is>
+      </c>
+      <c r="D283" s="14" t="inlineStr">
+        <is>
+          <t>https://www.penzionpribisko.sk</t>
+        </is>
+      </c>
+      <c r="E283" s="14" t="inlineStr">
+        <is>
+          <t>penzion@penzionpribisko.sk</t>
+        </is>
+      </c>
+      <c r="F283" s="13" t="inlineStr">
+        <is>
+          <t>+421 907 873 336</t>
+        </is>
+      </c>
+      <c r="G283" s="13" t="inlineStr">
+        <is>
+          <t>Zuberec (Roháče)</t>
+        </is>
+      </c>
+      <c r="H283" s="14" t="inlineStr">
+        <is>
+          <t>AI concierge, ktorý podľa termínu/počtu nocí odporučí balík a nasmeruje na online rezerváciu; SK aj PL</t>
+        </is>
+      </c>
+      <c r="I283" s="14" t="inlineStr">
+        <is>
+          <t>Guide sekcia 3 – veľa balíkov + viacjazyční (PL) hostia</t>
+        </is>
+      </c>
+      <c r="J283" s="13" t="inlineStr">
+        <is>
+          <t>Stredná</t>
+        </is>
+      </c>
+      <c r="K283" s="13" t="inlineStr">
+        <is>
+          <t>Draft pripravený</t>
+        </is>
+      </c>
+      <c r="L283" s="13" t="inlineStr"/>
+      <c r="M283" s="14" t="inlineStr">
+        <is>
+          <t>Wellness penzión v Zuberci, veľa balíkov (polpenzia+wellness, letné/zimné, apartmány), svadby, Gulash Fest. Web v SK/PL/EN, online rezervácia (Profitroom). Bez chatbota.</t>
+        </is>
+      </c>
+      <c r="N283" s="21" t="inlineStr"/>
+    </row>
+    <row r="284">
+      <c r="A284" s="13" t="n">
+        <v>323</v>
+      </c>
+      <c r="B284" s="13" t="inlineStr">
+        <is>
+          <t>Reality</t>
+        </is>
+      </c>
+      <c r="C284" s="14" t="inlineStr">
+        <is>
+          <t>GESTTO</t>
+        </is>
+      </c>
+      <c r="D284" s="14" t="inlineStr">
+        <is>
+          <t>https://www.gestto.sk</t>
+        </is>
+      </c>
+      <c r="E284" s="14" t="inlineStr">
+        <is>
+          <t>info@gestto.sk</t>
+        </is>
+      </c>
+      <c r="F284" s="13" t="inlineStr">
+        <is>
+          <t>+421 915 733 133</t>
+        </is>
+      </c>
+      <c r="G284" s="13" t="inlineStr">
+        <is>
+          <t>Trnava</t>
+        </is>
+      </c>
+      <c r="H284" s="14" t="inlineStr">
+        <is>
+          <t>AI lead qualifier – položí predávajúcemu základné otázky, spustí orientačné nacenenie a odovzdá kvalifikovaný lead</t>
+        </is>
+      </c>
+      <c r="I284" s="14" t="inlineStr">
+        <is>
+          <t>Guide sekcia 4 – kvalifikácia dopytov (Pre klientov hľadáme + nacenenie)</t>
+        </is>
+      </c>
+      <c r="J284" s="13" t="inlineStr">
+        <is>
+          <t>Stredná</t>
+        </is>
+      </c>
+      <c r="K284" s="13" t="inlineStr">
+        <is>
+          <t>Draft pripravený</t>
+        </is>
+      </c>
+      <c r="L284" s="13" t="inlineStr"/>
+      <c r="M284" s="14" t="inlineStr">
+        <is>
+          <t>Realitka v Trnave, tím 6 maklérov (Kopčová/Kopčo), sekcia 'Pre klientov hľadáme' + formulár na nacenenie. Silné recenzie na osobný prístup. Kontakt len cez formulár. Bez chatbota.</t>
+        </is>
+      </c>
+      <c r="N284" s="21" t="inlineStr"/>
+    </row>
+    <row r="285">
+      <c r="A285" s="13" t="n">
+        <v>324</v>
+      </c>
+      <c r="B285" s="13" t="inlineStr">
+        <is>
+          <t>Reality</t>
+        </is>
+      </c>
+      <c r="C285" s="14" t="inlineStr">
+        <is>
+          <t>NEOREAL</t>
+        </is>
+      </c>
+      <c r="D285" s="14" t="inlineStr">
+        <is>
+          <t>https://www.neoreal.sk</t>
+        </is>
+      </c>
+      <c r="E285" s="14" t="inlineStr">
+        <is>
+          <t>neoreal@neoreal.sk</t>
+        </is>
+      </c>
+      <c r="F285" s="13" t="inlineStr">
+        <is>
+          <t>+421 911 123 474</t>
+        </is>
+      </c>
+      <c r="G285" s="13" t="inlineStr">
+        <is>
+          <t>Trnava / Bratislava</t>
+        </is>
+      </c>
+      <c r="H285" s="14" t="inlineStr">
+        <is>
+          <t>AI asistent na otázky k developerským projektom (voľné byty, ceny, termín odovzdania) + zápis kvalifikovaného leadu 24/7</t>
+        </is>
+      </c>
+      <c r="I285" s="14" t="inlineStr">
+        <is>
+          <t>Guide sekcia 5 – konkrétnosť (menované projekty) + observácia (Lorem ipsum na webe)</t>
+        </is>
+      </c>
+      <c r="J285" s="13" t="inlineStr">
+        <is>
+          <t>Stredná</t>
+        </is>
+      </c>
+      <c r="K285" s="13" t="inlineStr">
+        <is>
+          <t>Draft pripravený</t>
+        </is>
+      </c>
+      <c r="L285" s="13" t="inlineStr"/>
+      <c r="M285" s="14" t="inlineStr">
+        <is>
+          <t>Etablovaná realitka (19 rokov), zameraná na developerské projekty (Cukrovar, ZicherHouse, Lakeside36), tím ~9. Kontakt len cez formulár, na hlavnej stránke ešte vzorový text 'Lorem ipsum'. Bez chatbota.</t>
+        </is>
+      </c>
+      <c r="N285" s="21" t="inlineStr"/>
+    </row>
+    <row r="286">
+      <c r="A286" s="13" t="n">
+        <v>325</v>
+      </c>
+      <c r="B286" s="13" t="inlineStr">
+        <is>
+          <t>E-shop</t>
+        </is>
+      </c>
+      <c r="C286" s="14" t="inlineStr">
+        <is>
+          <t>Herbex (HERBEX spol. s r.o.)</t>
+        </is>
+      </c>
+      <c r="D286" s="14" t="inlineStr">
+        <is>
+          <t>https://www.herbex.sk</t>
+        </is>
+      </c>
+      <c r="E286" s="14" t="inlineStr">
+        <is>
+          <t>info@herbex.sk</t>
+        </is>
+      </c>
+      <c r="F286" s="13" t="inlineStr">
+        <is>
+          <t>+421 32 77 421 12</t>
+        </is>
+      </c>
+      <c r="G286" s="13" t="inlineStr">
+        <is>
+          <t>Vinica</t>
+        </is>
+      </c>
+      <c r="H286" s="14" t="inlineStr">
+        <is>
+          <t>AI poradca, ktorý podľa symptómu („na pečeň“) odporučí konkrétny čaj z katalógu; obslúži aj B2B partnerov</t>
+        </is>
+      </c>
+      <c r="I286" s="14" t="inlineStr">
+        <is>
+          <t>Guide sekcia 3 – observácia z katalógu (čaje pomenované podľa indikácie) + jeden nápad</t>
+        </is>
+      </c>
+      <c r="J286" s="13" t="inlineStr">
+        <is>
+          <t>Vysoká</t>
+        </is>
+      </c>
+      <c r="K286" s="13" t="inlineStr">
+        <is>
+          <t>Draft pripravený</t>
+        </is>
+      </c>
+      <c r="L286" s="13" t="n"/>
+      <c r="M286" s="14" t="inlineStr">
+        <is>
+          <t>Rodinná firma od 1991, e-shop od 2017, vlastné pestovanie byliniek na Myjavských kopaniciach. Predávajú sypané/porciované/BIO/detské čaje, šumienky, psyllium, levanduľové výrobky. Čaje sú pomenované podľa indikácie (Pankreas a trávenie, Urologický čaj s brusnicami FORTE, Posilnená imunita ČAGA) – zákazník hľadá podľa problému, nie podľa názvu. Majú B2B portál 'Prihlásenie pre firmy' a samostatný CZ e-shop. Bez chatbota. Tón: vecný, edukatívny (blog o pestovaní).</t>
+        </is>
+      </c>
+      <c r="N286" s="21" t="n"/>
+    </row>
+    <row r="287">
+      <c r="A287" s="13" t="n">
+        <v>326</v>
+      </c>
+      <c r="B287" s="13" t="inlineStr">
+        <is>
+          <t>E-shop</t>
+        </is>
+      </c>
+      <c r="C287" s="14" t="inlineStr">
+        <is>
+          <t>HAKY-BAKY (Detský textil)</t>
+        </is>
+      </c>
+      <c r="D287" s="14" t="inlineStr">
+        <is>
+          <t>https://haky-baky.sk</t>
+        </is>
+      </c>
+      <c r="E287" s="14" t="inlineStr">
+        <is>
+          <t>info.hakybaky@gmail.com</t>
+        </is>
+      </c>
+      <c r="F287" s="13" t="inlineStr">
+        <is>
+          <t>+421 905 348 522</t>
+        </is>
+      </c>
+      <c r="G287" s="13" t="inlineStr">
+        <is>
+          <t>Martin</t>
+        </is>
+      </c>
+      <c r="H287" s="14" t="inlineStr">
+        <is>
+          <t>Sprievodca veľkosťami, ktorý zbiera miery dieťatka štruktúrovane pred objednávkou namiesto voľného textu v poznámke</t>
+        </is>
+      </c>
+      <c r="I287" s="14" t="inlineStr">
+        <is>
+          <t>Guide sekcia 3 – ostrá observácia z webu (úprava na mieru cez poznámku k objednávke)</t>
+        </is>
+      </c>
+      <c r="J287" s="13" t="inlineStr">
+        <is>
+          <t>Vysoká</t>
+        </is>
+      </c>
+      <c r="K287" s="13" t="inlineStr">
+        <is>
+          <t>Draft pripravený</t>
+        </is>
+      </c>
+      <c r="L287" s="13" t="n"/>
+      <c r="M287" s="14" t="inlineStr">
+        <is>
+          <t>Malá martinská manufaktúra, šijú detské oblečenie, 30 rokov na trhu, ocenenie Zlatá Firma. Kategórie: kojenecké, súpravy, vrchné, nohavice, spodná bielizeň, oblečenie na spanie, doplnky + dámske. KĽÚČOVÉ: na webe ponúkajú úpravu na mieru – zákazník napíše miery dieťatka do poznámky k objednávke (ručné spracovanie). Podpora len Po–Pi 8:00–16:30. Majú B2B veľkoobchodnú registráciu. Bez chatbota. Tón: vrelý, rodinný.</t>
+        </is>
+      </c>
+      <c r="N287" s="21" t="n"/>
+    </row>
+    <row r="288">
+      <c r="A288" s="13" t="n">
+        <v>327</v>
+      </c>
+      <c r="B288" s="13" t="inlineStr">
+        <is>
+          <t>E-shop</t>
+        </is>
+      </c>
+      <c r="C288" s="14" t="inlineStr">
+        <is>
+          <t>Amawell (klenotníctvo)</t>
+        </is>
+      </c>
+      <c r="D288" s="14" t="inlineStr">
+        <is>
+          <t>https://www.amawell.sk</t>
+        </is>
+      </c>
+      <c r="E288" s="14" t="inlineStr">
+        <is>
+          <t>info@amawell.sk</t>
+        </is>
+      </c>
+      <c r="F288" s="13" t="inlineStr">
+        <is>
+          <t>+421 910 233 222</t>
+        </is>
+      </c>
+      <c r="G288" s="13" t="inlineStr">
+        <is>
+          <t>Bratislava</t>
+        </is>
+      </c>
+      <c r="H288" s="14" t="inlineStr">
+        <is>
+          <t>Asistent, ktorý zákazníka s reklamáciou/servisom šperku nasmeruje na správnu predajňu namiesto výberu z 5 čísel a 3 mailov</t>
+        </is>
+      </c>
+      <c r="I288" s="14" t="inlineStr">
+        <is>
+          <t>Guide sekcia 3 – rozpor medzi sľubom (celoživotná starostlivosť) a roztriešteným kontaktom</t>
+        </is>
+      </c>
+      <c r="J288" s="13" t="inlineStr">
+        <is>
+          <t>Stredná</t>
+        </is>
+      </c>
+      <c r="K288" s="13" t="inlineStr">
+        <is>
+          <t>Draft pripravený</t>
+        </is>
+      </c>
+      <c r="L288" s="13" t="n"/>
+      <c r="M288" s="14" t="inlineStr">
+        <is>
+          <t>Klenotníctvo, zlaté a strieborné šperky, Magento e-shop + kamenné predajne (Aupark). Na webe sľubujú 'Garanciu celoživotnej starostlivosti zlatníka'. Kontaktná stránka má 5 telefónnych čísel a 3 e-maily (info@amawell.sk + adresy s doménou zendiamond.com) – zákazník nevie, kam sa obrátiť. Bez chatbota. Tón: vrelý, dôraz na kvalitu a dedičstvo. Používajú promo kódy (AMAWELL10).</t>
+        </is>
+      </c>
+      <c r="N288" s="21" t="n"/>
+    </row>
+    <row r="289">
+      <c r="A289" s="13" t="n">
+        <v>328</v>
+      </c>
+      <c r="B289" s="13" t="inlineStr">
+        <is>
+          <t>Zdravotníctvo</t>
+        </is>
+      </c>
+      <c r="C289" s="14" t="inlineStr">
+        <is>
+          <t>SKIN CARE s.r.o. (MUDr. Duchoňová)</t>
+        </is>
+      </c>
+      <c r="D289" s="14" t="inlineStr">
+        <is>
+          <t>https://www.duchonova.sk</t>
+        </is>
+      </c>
+      <c r="E289" s="14" t="inlineStr">
+        <is>
+          <t>strecnianska@duchonova.sk</t>
+        </is>
+      </c>
+      <c r="F289" s="13" t="inlineStr">
+        <is>
+          <t>+421 915 187 190</t>
+        </is>
+      </c>
+      <c r="G289" s="13" t="inlineStr">
+        <is>
+          <t>Bratislava-Petržalka</t>
+        </is>
+      </c>
+      <c r="H289" s="14" t="inlineStr">
+        <is>
+          <t>Asistent, ktorý pacienta nasmeruje na správny kanál (online poradňa / termín / dermatochirurgia) a súrne dopyty vyzdvihne navrch</t>
+        </is>
+      </c>
+      <c r="I289" s="14" t="inlineStr">
+        <is>
+          <t>Guide sekcia 4 – rezervácia roztrieštená medzi telefón, e-mail a navstevalekara.sk</t>
+        </is>
+      </c>
+      <c r="J289" s="13" t="inlineStr">
+        <is>
+          <t>Vysoká</t>
+        </is>
+      </c>
+      <c r="K289" s="13" t="inlineStr">
+        <is>
+          <t>Draft pripravený</t>
+        </is>
+      </c>
+      <c r="L289" s="13" t="n"/>
+      <c r="M289" s="14" t="inlineStr">
+        <is>
+          <t>Súkromná dermatovenerologická ambulancia pre deti aj dospelých, bez zmlúv so zdravotnými poisťovňami, netreba výmenný lístok. Ponúkajú aj online konzultáciu (telemedicína). PAIN POINT (recenzia na ich webe, zdroj navstevalekara.sk, pacientka Eva): 'Napriek tomu, že mala na mesiac dopredu úplne plno tak ma vzala hneď na druhy deň ako akútny prípad.' Objednávanie je rozdelené: telefón, e-mail, a navstevalekara.sk len pre časť lekárov. Bez chatbota.</t>
+        </is>
+      </c>
+      <c r="N289" s="21" t="n"/>
+    </row>
+    <row r="290">
+      <c r="A290" s="13" t="n">
+        <v>329</v>
+      </c>
+      <c r="B290" s="13" t="inlineStr">
+        <is>
+          <t>Zdravotníctvo</t>
+        </is>
+      </c>
+      <c r="C290" s="14" t="inlineStr">
+        <is>
+          <t>Rehabko (privátna ambulancia liečebnej rehabilitácie)</t>
+        </is>
+      </c>
+      <c r="D290" s="14" t="inlineStr">
+        <is>
+          <t>https://rehabko.sk</t>
+        </is>
+      </c>
+      <c r="E290" s="14" t="inlineStr">
+        <is>
+          <t>kotrbancova@rehabko.sk</t>
+        </is>
+      </c>
+      <c r="F290" s="13" t="inlineStr">
+        <is>
+          <t>+421 903 944 371</t>
+        </is>
+      </c>
+      <c r="G290" s="13" t="inlineStr">
+        <is>
+          <t>Žilina</t>
+        </is>
+      </c>
+      <c r="H290" s="14" t="inlineStr">
+        <is>
+          <t>Asistent, ktorý roztriedi dopyt (terapia vs. kurz), odpovie na bežné otázky a doručí kompletný zápis</t>
+        </is>
+      </c>
+      <c r="I290" s="14" t="inlineStr">
+        <is>
+          <t>Guide sekcia 3 – observácia z webu (kurzy cez Google Forms, žiadny rezervačný systém)</t>
+        </is>
+      </c>
+      <c r="J290" s="13" t="inlineStr">
+        <is>
+          <t>Stredná</t>
+        </is>
+      </c>
+      <c r="K290" s="13" t="inlineStr">
+        <is>
+          <t>Draft pripravený</t>
+        </is>
+      </c>
+      <c r="L290" s="13" t="n"/>
+      <c r="M290" s="14" t="inlineStr">
+        <is>
+          <t>Fyzioterapia pri bolestiach chrbtice, detská rehabilitácia, poúrazová rehabilitácia, kostrč a panvové dno, športová fyzioterapia. Používajú metódu McKenzie. Web na Squarespace. Žiadny rezervačný systém – kontakt len telefón/e-mail/formulár, prihlášky na kurzy cez Google Forms. Na kontakte je aj osobný Gmail (v drafte som to zámerne nespomínal). Bez chatbota. Tón: formálny, citáty (Goethe, Hippokrates).</t>
+        </is>
+      </c>
+      <c r="N290" s="21" t="n"/>
+    </row>
+    <row r="291">
+      <c r="A291" s="13" t="n">
+        <v>330</v>
+      </c>
+      <c r="B291" s="13" t="inlineStr">
+        <is>
+          <t>Zdravotníctvo</t>
+        </is>
+      </c>
+      <c r="C291" s="14" t="inlineStr">
+        <is>
+          <t>ORTOINOVA (ortopedická ambulancia)</t>
+        </is>
+      </c>
+      <c r="D291" s="14" t="inlineStr">
+        <is>
+          <t>https://ortoinova.sk</t>
+        </is>
+      </c>
+      <c r="E291" s="14" t="inlineStr">
+        <is>
+          <t>info@ortoinova.sk</t>
+        </is>
+      </c>
+      <c r="F291" s="13" t="inlineStr">
+        <is>
+          <t>+421 948 395 168</t>
+        </is>
+      </c>
+      <c r="G291" s="13" t="inlineStr">
+        <is>
+          <t>Bratislava-Ružinov</t>
+        </is>
+      </c>
+      <c r="H291" s="14" t="inlineStr">
+        <is>
+          <t>Asistent, ktorý pacienta zatriedi (USG / denzitometria / biologická liečba kĺbov) a rovno ponúkne termíny namiesto callbacku</t>
+        </is>
+      </c>
+      <c r="I291" s="14" t="inlineStr">
+        <is>
+          <t>Guide sekcia 3 – konkrétny bug na ich webe ako hook + free value v CTA</t>
+        </is>
+      </c>
+      <c r="J291" s="13" t="inlineStr">
+        <is>
+          <t>Vysoká</t>
+        </is>
+      </c>
+      <c r="K291" s="13" t="inlineStr">
+        <is>
+          <t>Draft pripravený</t>
+        </is>
+      </c>
+      <c r="L291" s="13" t="n"/>
+      <c r="M291" s="14" t="inlineStr">
+        <is>
+          <t>Ortopedická ambulancia, Zdravotné stredisko Trnávka. Ponuka: biologická liečba kĺbov, vyšetrenie pohybového aparátu, screeningová denzitometria, USG kĺbov dospelých aj bábätiek, viskosuplementy, laserová terapia. HOOK: na kontaktnej stránke je zobrazená adresa Info@ortoinova.sk, ale mailto odkaz vedie na info@pharco.sk – overené v HTML. POZOR: ak mail bounce-ne, skúsiť info@pharco.sk. Objednanie len cez callback formulár. Bez chatbota.</t>
+        </is>
+      </c>
+      <c r="N291" s="21" t="n"/>
+    </row>
+    <row r="292">
+      <c r="A292" s="13" t="n">
+        <v>331</v>
+      </c>
+      <c r="B292" s="13" t="inlineStr">
+        <is>
+          <t>Fitness/Wellness</t>
+        </is>
+      </c>
+      <c r="C292" s="14" t="inlineStr">
+        <is>
+          <t>Balance gym Žilina</t>
+        </is>
+      </c>
+      <c r="D292" s="14" t="inlineStr">
+        <is>
+          <t>https://balancegym.sk</t>
+        </is>
+      </c>
+      <c r="E292" s="14" t="inlineStr">
+        <is>
+          <t>info@balancegym.sk</t>
+        </is>
+      </c>
+      <c r="F292" s="13" t="inlineStr">
+        <is>
+          <t>+421 915 546 462</t>
+        </is>
+      </c>
+      <c r="G292" s="13" t="inlineStr">
+        <is>
+          <t>Žilina</t>
+        </is>
+      </c>
+      <c r="H292" s="14" t="inlineStr">
+        <is>
+          <t>Asistent, ktorý ukáže reálne voľné okná a rezerváciu doručí s kvalifikáciou klienta namiesto callbacku z formulára</t>
+        </is>
+      </c>
+      <c r="I292" s="14" t="inlineStr">
+        <is>
+          <t>Guide sekcia 3 – observácia z webu (otváracie hodiny „podľa rezervácií“)</t>
+        </is>
+      </c>
+      <c r="J292" s="13" t="inlineStr">
+        <is>
+          <t>Vysoká</t>
+        </is>
+      </c>
+      <c r="K292" s="13" t="inlineStr">
+        <is>
+          <t>Draft pripravený</t>
+        </is>
+      </c>
+      <c r="L292" s="13" t="n"/>
+      <c r="M292" s="14" t="inlineStr">
+        <is>
+          <t>Súkromné fitness centrum. Ponuka: individuálne aj skupinové tréningy, masáže a regenerácia (bankovanie, mäkké techniky), jedálničky na mieru, diagnostika InBody a VALD. HOOK: otváracie hodiny sú na webe uvedené doslova ako 'Pondelok – Nedeľa, podľa rezervácií' – klient nevie zistiť dostupnosť bez toho, aby napísal. Prvý tréning sa objednáva formulárom + callback. Bez chatbota. Tón: kamarátsky, tykanie ('u nás sa budeš cítiť ako doma').</t>
+        </is>
+      </c>
+      <c r="N292" s="21" t="n"/>
+    </row>
+    <row r="293">
+      <c r="A293" s="13" t="n">
+        <v>332</v>
+      </c>
+      <c r="B293" s="13" t="inlineStr">
+        <is>
+          <t>Fitness/Wellness</t>
+        </is>
+      </c>
+      <c r="C293" s="14" t="inlineStr">
+        <is>
+          <t>Gym75</t>
+        </is>
+      </c>
+      <c r="D293" s="14" t="inlineStr">
+        <is>
+          <t>https://gym75.sk</t>
+        </is>
+      </c>
+      <c r="E293" s="14" t="inlineStr">
+        <is>
+          <t>info@gym75.sk</t>
+        </is>
+      </c>
+      <c r="F293" s="13" t="inlineStr">
+        <is>
+          <t>+421 902 124 778</t>
+        </is>
+      </c>
+      <c r="G293" s="13" t="inlineStr">
+        <is>
+          <t>Bratislava-Ružinov</t>
+        </is>
+      </c>
+      <c r="H293" s="14" t="inlineStr">
+        <is>
+          <t>Asistent, ktorý odbaví výnimky mimo Gymify (storno Flex Passu, pokazený stroj, otázky na výbavu) bez telefonátu</t>
+        </is>
+      </c>
+      <c r="I293" s="14" t="inlineStr">
+        <is>
+          <t>Guide sekcia 3 – observácia z cenníka/FAQ + zrkadlenie ich tónu</t>
+        </is>
+      </c>
+      <c r="J293" s="13" t="inlineStr">
+        <is>
+          <t>Vysoká</t>
+        </is>
+      </c>
+      <c r="K293" s="13" t="inlineStr">
+        <is>
+          <t>Odoslané</t>
+        </is>
+      </c>
+      <c r="L293" s="13" t="inlineStr">
+        <is>
+          <t>16.07.2026</t>
+        </is>
+      </c>
+      <c r="M293" s="14" t="inlineStr">
+        <is>
+          <t>Súkromné samoobslužné fitness štúdio, bez recepcie. Rezervácia slotu, platba kartou a vstup cez QR – všetko cez externú appku Gymify. Ceny: jednorazový vstup 13€, mini 45€, standard 85€, pro 150€. Výbava: half rack, jednoručky 2,5–30 kg, kettlebells. HOOK: celý model je bezobslužný, ale výnimky (presun Flex Passu po 24h lehote, pokazený stroj) sa riešia telefónom/SMS/mailom. Bez chatbota. Tón: veľmi neformálny, tykanie ('Kupuješ si službu, nevstupuješ do manželstva!').</t>
+        </is>
+      </c>
+      <c r="N293" s="21" t="n"/>
+    </row>
+    <row r="294">
+      <c r="A294" s="13" t="n">
+        <v>333</v>
+      </c>
+      <c r="B294" s="13" t="inlineStr">
+        <is>
+          <t>Fitness/Wellness</t>
+        </is>
+      </c>
+      <c r="C294" s="14" t="inlineStr">
+        <is>
+          <t>Studio PL (cvičenie Košice)</t>
+        </is>
+      </c>
+      <c r="D294" s="14" t="inlineStr">
+        <is>
+          <t>https://cviceniekosice.sk</t>
+        </is>
+      </c>
+      <c r="E294" s="14" t="n"/>
+      <c r="F294" s="13" t="inlineStr">
+        <is>
+          <t>+421 948 006 659</t>
+        </is>
+      </c>
+      <c r="G294" s="13" t="inlineStr">
+        <is>
+          <t>Košice</t>
+        </is>
+      </c>
+      <c r="H294" s="14" t="inlineStr">
+        <is>
+          <t>Rozvrh aj rezervačný odkaz sú pochované v datovanom blogovom príspevku; potenciál na web + asistenta</t>
+        </is>
+      </c>
+      <c r="I294" s="14" t="inlineStr">
+        <is>
+          <t>Zatiaľ bez pitchu – chýba e-mail</t>
+        </is>
+      </c>
+      <c r="J294" s="13" t="inlineStr">
+        <is>
+          <t>Nízka</t>
+        </is>
+      </c>
+      <c r="K294" s="13" t="inlineStr">
+        <is>
+          <t>Email chýba</t>
+        </is>
+      </c>
+      <c r="L294" s="13" t="n"/>
+      <c r="M294" s="14" t="inlineStr">
+        <is>
+          <t>Skupinové cvičenia v Košiciach (CORE tréning, FYZIO lekcia, ZUMBA, FlexPower), kontaktná osoba Petra Lacková. Od jan. 2026 pôsobia v Elite Sport Centre, Uherova 13, Košice-Terasa (v pätičke je ešte stará adresa OC Luník II). Rezervácie cez externý isportsystem.sk, odkaz aj rozvrh sú len vnútri starého blogového príspevku. NA WEBE NIE JE ŽIADNY E-MAIL – dopyty idú na jeden mobil. Bez chatbota. Draft nevytvorený. Ďalší krok: dohľadať e-mail cez FB/IG alebo zavolať.</t>
+        </is>
+      </c>
+      <c r="N294" s="21" t="n"/>
+    </row>
+    <row r="295">
+      <c r="A295" s="13" t="n">
+        <v>334</v>
+      </c>
+      <c r="B295" s="13" t="inlineStr">
+        <is>
+          <t>Gastro</t>
+        </is>
+      </c>
+      <c r="C295" s="14" t="inlineStr">
+        <is>
+          <t>Quo Vadis Reštaurácia</t>
+        </is>
+      </c>
+      <c r="D295" s="14" t="inlineStr">
+        <is>
+          <t>https://quovadisnitra.sk</t>
+        </is>
+      </c>
+      <c r="E295" s="14" t="inlineStr">
+        <is>
+          <t>info@quovadisnitra.sk</t>
+        </is>
+      </c>
+      <c r="F295" s="13" t="inlineStr">
+        <is>
+          <t>+421 918 253 276</t>
+        </is>
+      </c>
+      <c r="G295" s="13" t="inlineStr">
+        <is>
+          <t>Nitra (Zobor)</t>
+        </is>
+      </c>
+      <c r="H295" s="14" t="inlineStr">
+        <is>
+          <t>Asistent, ktorý zoberie rezerváciu aj mimo 10:00–22:00 a odpovie na týždenné menu bez duplicitnej správy obsahu</t>
+        </is>
+      </c>
+      <c r="I295" s="14" t="inlineStr">
+        <is>
+          <t>Guide sekcia 4 – rezervácie mimo otváracích hodín (vzor pre reštaurácie)</t>
+        </is>
+      </c>
+      <c r="J295" s="13" t="inlineStr">
+        <is>
+          <t>Stredná</t>
+        </is>
+      </c>
+      <c r="K295" s="13" t="inlineStr">
+        <is>
+          <t>Draft pripravený</t>
+        </is>
+      </c>
+      <c r="L295" s="13" t="n"/>
+      <c r="M295" s="14" t="inlineStr">
+        <is>
+          <t>Reštaurácia na Zobore. Ponuka: A'la Carte, týždenné menu, catering pre firmy aj súkromné podujatia, moderná medzinárodná kuchyňa. HOOK: rezervačný formulár na /rezervacia/ existuje, ale hlavná stránka posiela hostí telefonovať medzi 10:00–22:00. Týždenné menu je samostatná stránka, ktorú treba ručne prepisovať. Recenzie posielajú na Google. Bez chatbota. Tón: elegantný, aspiračný ('Vaša cesta za kulinárskym zážitkom').</t>
+        </is>
+      </c>
+      <c r="N295" s="21" t="n"/>
+    </row>
+    <row r="296">
+      <c r="A296" s="13" t="n">
+        <v>335</v>
+      </c>
+      <c r="B296" s="13" t="inlineStr">
+        <is>
+          <t>Hotel/Penzión</t>
+        </is>
+      </c>
+      <c r="C296" s="14" t="inlineStr">
+        <is>
+          <t>Penzión Slovakia</t>
+        </is>
+      </c>
+      <c r="D296" s="14" t="inlineStr">
+        <is>
+          <t>https://penzion-slovakia.sk</t>
+        </is>
+      </c>
+      <c r="E296" s="14" t="inlineStr">
+        <is>
+          <t>penzionslovakia@gmail.com</t>
+        </is>
+      </c>
+      <c r="F296" s="13" t="inlineStr">
+        <is>
+          <t>+421 904 064 492</t>
+        </is>
+      </c>
+      <c r="G296" s="13" t="inlineStr">
+        <is>
+          <t>Ždiar (Belianske Tatry)</t>
+        </is>
+      </c>
+      <c r="H296" s="14" t="inlineStr">
+        <is>
+          <t>Asistent s reálnou dostupnosťou izieb a cenou s raňajkami; do mailu len dopyty vyžadujúce rozhodnutie (skupiny, bicykle, mikrobus)</t>
+        </is>
+      </c>
+      <c r="I296" s="14" t="inlineStr">
+        <is>
+          <t>Guide sekcia 4 – rezervačné CTA vedú len na nezáväzný dopyt</t>
+        </is>
+      </c>
+      <c r="J296" s="13" t="inlineStr">
+        <is>
+          <t>Vysoká</t>
+        </is>
+      </c>
+      <c r="K296" s="13" t="inlineStr">
+        <is>
+          <t>Odoslané</t>
+        </is>
+      </c>
+      <c r="L296" s="13" t="inlineStr">
+        <is>
+          <t>14.07.2026</t>
+        </is>
+      </c>
+      <c r="M296" s="14" t="inlineStr">
+        <is>
+          <t>Celoročný penzión v Ždiari, majiteľ Dušan Pirog. Kapacita 40 lôžok (uvedené na ich webe). Izby: apartmán, dvojlôžková, štúdio, trojlôžková; balkón pri každej izbe. Goralská reštaurácia (halušky, pirohy), požičovňa bicyklov, mini bus-taxi. Ceny od 30 €/os./noc, raňajky 10 €. HOOK: všetky tlačidlá 'Rezervovať online' vedú len na nezáväzný dopytový formulár, žiadny kalendár. Navyše mailto v hlavičke vedie na info@penzionslovakia.sk, hoci zobrazená adresa je gmail. Bez chatbota.</t>
+        </is>
+      </c>
+      <c r="N296" s="21" t="n"/>
+    </row>
+    <row r="297">
+      <c r="A297" s="13" t="n">
+        <v>336</v>
+      </c>
+      <c r="B297" s="13" t="inlineStr">
+        <is>
+          <t>Hotel/Penzión</t>
+        </is>
+      </c>
+      <c r="C297" s="14" t="inlineStr">
+        <is>
+          <t>Penzión u Hanky</t>
+        </is>
+      </c>
+      <c r="D297" s="14" t="inlineStr">
+        <is>
+          <t>https://www.penzionuhanky.sk</t>
+        </is>
+      </c>
+      <c r="E297" s="14" t="inlineStr">
+        <is>
+          <t>info@ubytovanietelgart.sk</t>
+        </is>
+      </c>
+      <c r="F297" s="13" t="inlineStr">
+        <is>
+          <t>+421 903 771 662</t>
+        </is>
+      </c>
+      <c r="G297" s="13" t="inlineStr">
+        <is>
+          <t>Telgárt</t>
+        </is>
+      </c>
+      <c r="H297" s="14" t="inlineStr">
+        <is>
+          <t>Dopísať vlastný rezervačný systém do slovenčiny + asistent na opakované otázky (parkovanie, raňajky, wifi, okolie)</t>
+        </is>
+      </c>
+      <c r="I297" s="14" t="inlineStr">
+        <is>
+          <t>Guide sekcia 3 – veľmi konkrétna chyba v rezervačnom flow</t>
+        </is>
+      </c>
+      <c r="J297" s="13" t="inlineStr">
+        <is>
+          <t>Vysoká</t>
+        </is>
+      </c>
+      <c r="K297" s="13" t="inlineStr">
+        <is>
+          <t>Odoslané</t>
+        </is>
+      </c>
+      <c r="L297" s="13" t="inlineStr">
+        <is>
+          <t>14.07.2026</t>
+        </is>
+      </c>
+      <c r="M297" s="14" t="inlineStr">
+        <is>
+          <t>Penzión pri lyžiarskom stredisku Telgárt, 9 izieb / 24 lôžok. Dvojposteľová od 65 €, trojposteľová od 80 €, štvorposteľová od 90 €. Vlastná kúpeľňa, TV, wifi, páperové/protialergické periny. Reštaurácia + bar so slovenskými a českými vínami od malých vinárov. HOOK: majú vlastný rezervačný systém (WordPress Hotale/Tourmaster), ale checkout sa prepne do angličtiny a používa formulácie pre zájazdy – 'you can also rate the tour after you finished the tour'. Bez chatbota. Tón: vrelý ('Varíme tak, ako by sme varili sami pre seba').</t>
+        </is>
+      </c>
+      <c r="N297" s="21" t="n"/>
+    </row>
+    <row r="298">
+      <c r="A298" s="13" t="n">
+        <v>337</v>
+      </c>
+      <c r="B298" s="13" t="inlineStr">
+        <is>
+          <t>Hotel/Penzión</t>
+        </is>
+      </c>
+      <c r="C298" s="14" t="inlineStr">
+        <is>
+          <t>Penzión Raj</t>
+        </is>
+      </c>
+      <c r="D298" s="14" t="inlineStr">
+        <is>
+          <t>https://penzionraj.sk</t>
+        </is>
+      </c>
+      <c r="E298" s="14" t="inlineStr">
+        <is>
+          <t>info@penzionraj.sk</t>
+        </is>
+      </c>
+      <c r="F298" s="13" t="inlineStr">
+        <is>
+          <t>+421 917 681 326</t>
+        </is>
+      </c>
+      <c r="G298" s="13" t="inlineStr">
+        <is>
+          <t>Rajecké Teplice</t>
+        </is>
+      </c>
+      <c r="H298" s="14" t="inlineStr">
+        <is>
+          <t>Nový mobilný web + asistent s dostupnosťou izieb a tipmi na okolie (kúpalisko v lete, zjazdovky v zime)</t>
+        </is>
+      </c>
+      <c r="I298" s="14" t="inlineStr">
+        <is>
+          <t>Guide sekcia 3 – žiadny kalendár voľnosti, zastaraný web</t>
+        </is>
+      </c>
+      <c r="J298" s="13" t="inlineStr">
+        <is>
+          <t>Stredná</t>
+        </is>
+      </c>
+      <c r="K298" s="13" t="inlineStr">
+        <is>
+          <t>Odoslané</t>
+        </is>
+      </c>
+      <c r="L298" s="13" t="inlineStr">
+        <is>
+          <t>14.07.2026</t>
+        </is>
+      </c>
+      <c r="M298" s="14" t="inlineStr">
+        <is>
+          <t>Penzión v Rajeckých Tepliciach (kúpeľné mesto). Sekcie: Izby, Reštaurácia, Cenník. Propagujú termálne kúpaliská a zimné športy v okolí. HOOK: žiadna online rezervácia ani kalendár – 'Ak máte záujem o rezerváciu... kontaktujte nás' + formulár na meno/adresu/telefón. Web je viditeľne zastaraný (pätička ©2014, fotky z 2013/2014). Bez chatbota. Tón: formálny, zdvorilý. Nižšia priorita – malý rozpočet, ale hook je jasný a zákazka by bola web + bot.</t>
+        </is>
+      </c>
+      <c r="N298" s="21" t="n"/>
+    </row>
+    <row r="299">
+      <c r="A299" s="13" t="n">
+        <v>338</v>
+      </c>
+      <c r="B299" s="13" t="inlineStr">
+        <is>
+          <t>Reality</t>
+        </is>
+      </c>
+      <c r="C299" s="14" t="inlineStr">
+        <is>
+          <t>Liniem Reality (Liniem s.r.o.)</t>
+        </is>
+      </c>
+      <c r="D299" s="14" t="inlineStr">
+        <is>
+          <t>https://www.liniemreality.sk</t>
+        </is>
+      </c>
+      <c r="E299" s="14" t="inlineStr">
+        <is>
+          <t>info@liniemreality.sk</t>
+        </is>
+      </c>
+      <c r="F299" s="13" t="inlineStr">
+        <is>
+          <t>+421 948 571 309</t>
+        </is>
+      </c>
+      <c r="G299" s="13" t="inlineStr">
+        <is>
+          <t>Nitra</t>
+        </is>
+      </c>
+      <c r="H299" s="14" t="inlineStr">
+        <is>
+          <t>Viacjazyčný AI lead qualifier k sekcii „Ponúknite nám“, ktorý dopyt smeruje maklérovi podľa lokality a jazyka</t>
+        </is>
+      </c>
+      <c r="I299" s="14" t="inlineStr">
+        <is>
+          <t>Guide sekcia 3 – rozpor: makléri majú vypísané jazyky, web je len po slovensky</t>
+        </is>
+      </c>
+      <c r="J299" s="13" t="inlineStr">
+        <is>
+          <t>Vysoká</t>
+        </is>
+      </c>
+      <c r="K299" s="13" t="inlineStr">
+        <is>
+          <t>Odoslané</t>
+        </is>
+      </c>
+      <c r="L299" s="13" t="inlineStr">
+        <is>
+          <t>14.07.2026</t>
+        </is>
+      </c>
+      <c r="M299" s="14" t="inlineStr">
+        <is>
+          <t>Realitka v Nitre (Staničná 7/A), CEO Peter Čoros RSc., tím 6 maklérov. Značka 'maklér so srdcom' (FB/IG). Služby: hypotekárne centrum, video obhliadka, dron, banery, open house. HOOK: pri každom maklérovi sú vypísané jazyky (Čoros Abaháziová – maďarsky; Konček – nemecky, taliansky; Kryvenko – ukrajinsky; Mihalčinová – poľsky), ale samotný web je len po slovensky. Ponuky majú aj mimo Nitry – Sereď, Košice, Prešov, Vysoké Tatry. Kontakt cez formulár 'Ponúknite nám'. Bez chatbota.</t>
+        </is>
+      </c>
+      <c r="N299" s="21" t="n"/>
+    </row>
+    <row r="300">
+      <c r="A300" s="13" t="n">
+        <v>339</v>
+      </c>
+      <c r="B300" s="13" t="inlineStr">
+        <is>
+          <t>Reality</t>
+        </is>
+      </c>
+      <c r="C300" s="14" t="inlineStr">
+        <is>
+          <t>Reality KONTAKT</t>
+        </is>
+      </c>
+      <c r="D300" s="14" t="inlineStr">
+        <is>
+          <t>https://www.reality-kontakt.sk</t>
+        </is>
+      </c>
+      <c r="E300" s="14" t="inlineStr">
+        <is>
+          <t>info@reality-kontakt.sk</t>
+        </is>
+      </c>
+      <c r="F300" s="13" t="inlineStr">
+        <is>
+          <t>+421 910 180 222</t>
+        </is>
+      </c>
+      <c r="G300" s="13" t="inlineStr">
+        <is>
+          <t>Nové Zámky</t>
+        </is>
+      </c>
+      <c r="H300" s="14" t="inlineStr">
+        <is>
+          <t>Asistent priamo pri ponuke: zistí kúpa/predaj, potrebu hypotéky a posudku, odovzdá maklérovi; vie aj po maďarsky</t>
+        </is>
+      </c>
+      <c r="I300" s="14" t="inlineStr">
+        <is>
+          <t>Guide sekcia 3 – rozbitý e-mailový odkaz v hlavičke ako hook</t>
+        </is>
+      </c>
+      <c r="J300" s="13" t="inlineStr">
+        <is>
+          <t>Vysoká</t>
+        </is>
+      </c>
+      <c r="K300" s="13" t="inlineStr">
+        <is>
+          <t>Odoslané</t>
+        </is>
+      </c>
+      <c r="L300" s="13" t="inlineStr">
+        <is>
+          <t>14.07.2026</t>
+        </is>
+      </c>
+      <c r="M300" s="14" t="inlineStr">
+        <is>
+          <t>Realitka v Nových Zámkoch, člen ZRKS. Sprostredkovanie predaja/kúpy/prenájmu (byty, domy, chaty, pozemky), poradenstvo pri tvorbe trhovej ceny, kompletný právny servis, legalizácia stavieb, nízke provízie. Dvojjazyčná SK + HU verzia (ingatlan.reality-kontakt.sk). HOOK: e-mail maczko@reality-kontakt.sk v hlavičke je zabalený v odkaze typu tel: – na mobile otvorí volanie namiesto mailu; pole 'Tel.:' v pätičke je prázdne. Pri ponukách posielajú volať na rôzne čísla. Bez chatbota. Tón: kamarátsky-profesionálny ('Príďte na kávu a poraďte sa').</t>
+        </is>
+      </c>
+      <c r="N300" s="21" t="n"/>
+    </row>
+    <row r="301">
+      <c r="A301" s="13" t="n">
+        <v>340</v>
+      </c>
+      <c r="B301" s="13" t="inlineStr">
+        <is>
+          <t>Reality</t>
+        </is>
+      </c>
+      <c r="C301" s="14" t="inlineStr">
+        <is>
+          <t>Trnava Reality</t>
+        </is>
+      </c>
+      <c r="D301" s="14" t="inlineStr">
+        <is>
+          <t>https://www.trnavareality.sk</t>
+        </is>
+      </c>
+      <c r="E301" s="14" t="inlineStr">
+        <is>
+          <t>trnavareality@trnavareality.sk</t>
+        </is>
+      </c>
+      <c r="F301" s="13" t="inlineStr">
+        <is>
+          <t>+421 904 903 903</t>
+        </is>
+      </c>
+      <c r="G301" s="13" t="inlineStr">
+        <is>
+          <t>Trnava</t>
+        </is>
+      </c>
+      <c r="H301" s="14" t="inlineStr">
+        <is>
+          <t>Dočistiť web + asistent pri sekcii „Chcem predať“, ktorý prevedie majiteľa otázkami a doručí kvalifikovaný lead</t>
+        </is>
+      </c>
+      <c r="I301" s="14" t="inlineStr">
+        <is>
+          <t>Guide sekcia 3 – zvyšky demo šablóny na webe ako hook</t>
+        </is>
+      </c>
+      <c r="J301" s="13" t="inlineStr">
+        <is>
+          <t>Vysoká</t>
+        </is>
+      </c>
+      <c r="K301" s="13" t="inlineStr">
+        <is>
+          <t>Odoslané</t>
+        </is>
+      </c>
+      <c r="L301" s="13" t="inlineStr">
+        <is>
+          <t>14.07.2026</t>
+        </is>
+      </c>
+      <c r="M301" s="14" t="inlineStr">
+        <is>
+          <t>Realitka v Trnave (Kapitulská 20), konateľ Mgr. Tomáš Málik, kolegyňa Mgr. Aneta Štefanovská (kancelaria@trnavareality.sk). Predaj/prenájom, developerské projekty, oceňovanie nehnuteľností. HOOK: na slovenskom webe zostali zvyšky demo šablóny – prihlasovací modal hlási 'User registration is disabled for demo purpose.' a v UI sú anglické 'Compare listings', 'Lost your password?'. Kontakt len cez formulár 'Napíšte nám'. Bez chatbota. Tón: upokojujúci, formálny.</t>
+        </is>
+      </c>
+      <c r="N301" s="21" t="n"/>
+    </row>
+    <row r="302">
+      <c r="A302" s="10" t="n">
+        <v>341</v>
+      </c>
+      <c r="B302" s="10" t="inlineStr">
+        <is>
+          <t>E-shop</t>
+        </is>
+      </c>
+      <c r="C302" s="10" t="inlineStr">
+        <is>
+          <t>Bioshop.sk (MOOIA s.r.o.)</t>
+        </is>
+      </c>
+      <c r="D302" s="10" t="inlineStr">
+        <is>
+          <t>https://www.bioshop.sk</t>
+        </is>
+      </c>
+      <c r="E302" s="10" t="inlineStr">
+        <is>
+          <t>info@bioshop.sk</t>
+        </is>
+      </c>
+      <c r="F302" s="10" t="inlineStr">
+        <is>
+          <t>+421 947 921 991</t>
+        </is>
+      </c>
+      <c r="G302" s="10" t="inlineStr">
+        <is>
+          <t>Slovensko (online)</t>
+        </is>
+      </c>
+      <c r="H302" s="10" t="inlineStr">
+        <is>
+          <t>AI poradca na webe podľa zdravotnej ťažkosti navedie zákazníka na konkrétnu bylinku/značku z katalógu; človeku nechá len odborné otázky</t>
+        </is>
+      </c>
+      <c r="I302" s="10" t="inlineStr">
+        <is>
+          <t>Observácia z webu: 'Bylinková poradňa – napíšte nám' + katalóg podľa problému</t>
+        </is>
+      </c>
+      <c r="J302" s="10" t="inlineStr">
+        <is>
+          <t>Vysoká</t>
+        </is>
+      </c>
+      <c r="K302" s="10" t="inlineStr">
+        <is>
+          <t>Odoslané</t>
+        </is>
+      </c>
+      <c r="L302" s="10" t="inlineStr">
+        <is>
+          <t>16.07.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" s="10" t="n">
+        <v>342</v>
+      </c>
+      <c r="B303" s="10" t="inlineStr">
+        <is>
+          <t>E-shop</t>
+        </is>
+      </c>
+      <c r="C303" s="10" t="inlineStr">
+        <is>
+          <t>Herbatica.sk</t>
+        </is>
+      </c>
+      <c r="D303" s="10" t="inlineStr">
+        <is>
+          <t>https://www.herbatica.sk</t>
+        </is>
+      </c>
+      <c r="E303" s="10" t="inlineStr">
+        <is>
+          <t>ahoj@herbatica.sk</t>
+        </is>
+      </c>
+      <c r="F303" s="10" t="inlineStr">
+        <is>
+          <t>+421 2/321 123 45</t>
+        </is>
+      </c>
+      <c r="G303" s="10" t="inlineStr">
+        <is>
+          <t>Piešťany + online (SK/CZ/HU/RO)</t>
+        </is>
+      </c>
+      <c r="H303" s="10" t="inlineStr">
+        <is>
+          <t>AI poradca odpovie na opakované otázky o zložení/vhodnosti (aj večer/víkend), odporučí produkt z 1000+, citlivé pošle na človeka</t>
+        </is>
+      </c>
+      <c r="I303" s="10" t="inlineStr">
+        <is>
+          <t>Observácia: navigácia 'Trápi ma' podľa ťažkostí + otázky zákazníkov pod produktmi</t>
+        </is>
+      </c>
+      <c r="J303" s="10" t="inlineStr">
+        <is>
+          <t>Vysoká</t>
+        </is>
+      </c>
+      <c r="K303" s="10" t="inlineStr">
+        <is>
+          <t>Odoslané</t>
+        </is>
+      </c>
+      <c r="L303" s="10" t="inlineStr">
+        <is>
+          <t>16.07.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" s="10" t="n">
+        <v>343</v>
+      </c>
+      <c r="B304" s="10" t="inlineStr">
+        <is>
+          <t>Zdravotníctvo</t>
+        </is>
+      </c>
+      <c r="C304" s="10" t="inlineStr">
+        <is>
+          <t>Kapadent, s.r.o. (zubná ambulancia)</t>
+        </is>
+      </c>
+      <c r="D304" s="10" t="inlineStr">
+        <is>
+          <t>https://kapadent.sk</t>
+        </is>
+      </c>
+      <c r="E304" s="10" t="inlineStr">
+        <is>
+          <t>kapadent.sro@gmail.com</t>
+        </is>
+      </c>
+      <c r="F304" s="10" t="inlineStr">
+        <is>
+          <t>+421 948 370 604</t>
+        </is>
+      </c>
+      <c r="G304" s="10" t="inlineStr">
+        <is>
+          <t>Čaňa pri Košiciach</t>
+        </is>
+      </c>
+      <c r="H304" s="10" t="inlineStr">
+        <is>
+          <t>AI booking bot 24/7 na web+IG prijme žiadosť o termín mimo hodín, spýta sa na dôvod, ráno pošle zoznam vrátane akútnych</t>
+        </is>
+      </c>
+      <c r="I304" s="10" t="inlineStr">
+        <is>
+          <t>Observácia: objednanie iba tel/formulár, ambulancia Po-Pia len do 15:30</t>
+        </is>
+      </c>
+      <c r="J304" s="10" t="inlineStr">
+        <is>
+          <t>Vysoká</t>
+        </is>
+      </c>
+      <c r="K304" s="10" t="inlineStr">
+        <is>
+          <t>Odoslané</t>
+        </is>
+      </c>
+      <c r="L304" s="10" t="inlineStr">
+        <is>
+          <t>16.07.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" s="10" t="n">
+        <v>344</v>
+      </c>
+      <c r="B305" s="10" t="inlineStr">
+        <is>
+          <t>Zdravotníctvo</t>
+        </is>
+      </c>
+      <c r="C305" s="10" t="inlineStr">
+        <is>
+          <t>MDDr. Dušan Škrobánek (Zubár Nitra)</t>
+        </is>
+      </c>
+      <c r="D305" s="10" t="inlineStr">
+        <is>
+          <t>https://www.zubar-nitra.sk</t>
+        </is>
+      </c>
+      <c r="E305" s="10" t="inlineStr">
+        <is>
+          <t>info@zubar-nitra.sk</t>
+        </is>
+      </c>
+      <c r="F305" s="10" t="inlineStr">
+        <is>
+          <t>0949 504 134</t>
+        </is>
+      </c>
+      <c r="G305" s="10" t="inlineStr">
+        <is>
+          <t>Nitra (Kalinčiakova 11)</t>
+        </is>
+      </c>
+      <c r="H305" s="10" t="inlineStr">
+        <is>
+          <t>AI bot prijme žiadosť o termín kedykoľvek, odlíši nového/objednaného pacienta a akútnu bolesť od prehliadky, ráno doručí prehľad</t>
+        </is>
+      </c>
+      <c r="I305" s="10" t="inlineStr">
+        <is>
+          <t>Observácia: rezervačný formulár + web 'momentálne zatvorené' večer aj víkend</t>
+        </is>
+      </c>
+      <c r="J305" s="10" t="inlineStr">
+        <is>
+          <t>Vysoká</t>
+        </is>
+      </c>
+      <c r="K305" s="10" t="inlineStr">
+        <is>
+          <t>Odoslané</t>
+        </is>
+      </c>
+      <c r="L305" s="10" t="inlineStr">
+        <is>
+          <t>16.07.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="10" t="n">
+        <v>345</v>
+      </c>
+      <c r="B306" s="10" t="inlineStr">
+        <is>
+          <t>Fitness/Wellness</t>
+        </is>
+      </c>
+      <c r="C306" s="10" t="inlineStr">
+        <is>
+          <t>Art of Pilates Studio</t>
+        </is>
+      </c>
+      <c r="D306" s="10" t="inlineStr">
+        <is>
+          <t>https://www.artofpilates.sk</t>
+        </is>
+      </c>
+      <c r="E306" s="10" t="inlineStr">
+        <is>
+          <t>info@artofpilates.sk</t>
+        </is>
+      </c>
+      <c r="F306" s="10" t="inlineStr">
+        <is>
+          <t>+421 910 957 424</t>
+        </is>
+      </c>
+      <c r="G306" s="10" t="inlineStr">
+        <is>
+          <t>Bratislava (Karlova Ves)</t>
+        </is>
+      </c>
+      <c r="H306" s="10" t="inlineStr">
+        <is>
+          <t>AI/WhatsApp asistent prevedie NOVÉHO klienta prvou rezerváciou aj večer, odporučí Indi/Duo alebo Reformer group a navrhne termín</t>
+        </is>
+      </c>
+      <c r="I306" s="10" t="inlineStr">
+        <is>
+          <t>Observácia: existujúci klient booking online, ale nový klient len telefonicky</t>
+        </is>
+      </c>
+      <c r="J306" s="10" t="inlineStr">
+        <is>
+          <t>Vysoká</t>
+        </is>
+      </c>
+      <c r="K306" s="10" t="inlineStr">
+        <is>
+          <t>Odoslané</t>
+        </is>
+      </c>
+      <c r="L306" s="10" t="inlineStr">
+        <is>
+          <t>16.07.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" s="10" t="n">
+        <v>346</v>
+      </c>
+      <c r="B307" s="10" t="inlineStr">
+        <is>
+          <t>Gastro</t>
+        </is>
+      </c>
+      <c r="C307" s="10" t="inlineStr">
+        <is>
+          <t>Bosco restaurant &amp; bowling</t>
+        </is>
+      </c>
+      <c r="D307" s="10" t="inlineStr">
+        <is>
+          <t>https://bosco.sk</t>
+        </is>
+      </c>
+      <c r="E307" s="10" t="inlineStr">
+        <is>
+          <t>boscorestaurant@gmail.com</t>
+        </is>
+      </c>
+      <c r="F307" s="10" t="inlineStr">
+        <is>
+          <t>0948 092 033</t>
+        </is>
+      </c>
+      <c r="G307" s="10" t="inlineStr">
+        <is>
+          <t>Trenčín</t>
+        </is>
+      </c>
+      <c r="H307" s="10" t="inlineStr">
+        <is>
+          <t>AI asistent k rezervácii stolov pridá dostupnosť bowlingových dráh + prvotné dopyty na oslavy/firemné akcie (počet, termín, detský kútik)</t>
+        </is>
+      </c>
+      <c r="I307" s="10" t="inlineStr">
+        <is>
+          <t>Observácia: stôl online (Bookio), ale bowling a oslavy len cez telefón</t>
+        </is>
+      </c>
+      <c r="J307" s="10" t="inlineStr">
+        <is>
+          <t>Stredná</t>
+        </is>
+      </c>
+      <c r="K307" s="10" t="inlineStr">
+        <is>
+          <t>Draft pripravený</t>
+        </is>
+      </c>
+      <c r="L307" s="10" t="inlineStr">
+        <is>
+          <t>Reštaurácia + bowling, 11 rokov, medzinárodná kuchyňa. Stoly cez Bookio Pro, ale bowling a firemné akcie/oslavy vybavujú telefonicky. Detský kútik, rozvoz denného menu. Recenzie na webe 5/5. Tón: rodinný, moderný.</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" s="10" t="n">
+        <v>347</v>
+      </c>
+      <c r="B308" s="10" t="inlineStr">
+        <is>
+          <t>Hotel/Penzión</t>
+        </is>
+      </c>
+      <c r="C308" s="10" t="inlineStr">
+        <is>
+          <t>Penzión Zuberec</t>
+        </is>
+      </c>
+      <c r="D308" s="10" t="inlineStr">
+        <is>
+          <t>https://zuberec.eu</t>
+        </is>
+      </c>
+      <c r="E308" s="10" t="inlineStr">
+        <is>
+          <t>penzion@zuberec.eu</t>
+        </is>
+      </c>
+      <c r="F308" s="10" t="inlineStr">
+        <is>
+          <t>+421 907 39 40 30</t>
+        </is>
+      </c>
+      <c r="G308" s="10" t="inlineStr">
+        <is>
+          <t>Zuberec (Roháče, Záp. Tatry)</t>
+        </is>
+      </c>
+      <c r="H308" s="10" t="inlineStr">
+        <is>
+          <t>AI asistent na web prijme dopyt o termín aj v noci + odpovie na FAQ (sauna, čo je zdarma, tipy na Roháče); alt. redesign webu s rezerváciou</t>
+        </is>
+      </c>
+      <c r="I308" s="10" t="inlineStr">
+        <is>
+          <t>Observácia: rezervácia iba tel/e-mail, web z r. 2014 bez rezervačného systému</t>
+        </is>
+      </c>
+      <c r="J308" s="10" t="inlineStr">
+        <is>
+          <t>Stredná</t>
+        </is>
+      </c>
+      <c r="K308" s="10" t="inlineStr">
+        <is>
+          <t>Draft pripravený</t>
+        </is>
+      </c>
+      <c r="L308" s="10" t="inlineStr">
+        <is>
+          <t>Rodinný penzión, celoročne. Web z 2014 (.php), rezervácia iba telefón/e-mail = hosť čaká na odpoveď. Veľa free služieb (wifi, biliard, altánok), sauna spoplatnená. Na webe tipy na výlety/lyžovačky. Tón: srdečný, rodinný.</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" s="10" t="n">
+        <v>348</v>
+      </c>
+      <c r="B309" s="10" t="inlineStr">
+        <is>
+          <t>Reality</t>
+        </is>
+      </c>
+      <c r="C309" s="10" t="inlineStr">
+        <is>
+          <t>Newcastle Reality s.r.o.</t>
+        </is>
+      </c>
+      <c r="D309" s="10" t="inlineStr">
+        <is>
+          <t>https://www.newcastle.sk</t>
+        </is>
+      </c>
+      <c r="E309" s="10" t="inlineStr">
+        <is>
+          <t>info@newcastle.sk</t>
+        </is>
+      </c>
+      <c r="F309" s="10" t="inlineStr">
+        <is>
+          <t>+421 904 543 210</t>
+        </is>
+      </c>
+      <c r="G309" s="10" t="inlineStr">
+        <is>
+          <t>Banská Bystrica</t>
+        </is>
+      </c>
+      <c r="H309" s="10" t="inlineStr">
+        <is>
+          <t>AI lead-qualifier na formulár 'Dopyt' sa pred maklérom spýta rozpočet, lokalitu, financovanie a dodá roztriedené dopyty s vážnymi navrchu</t>
+        </is>
+      </c>
+      <c r="I309" s="10" t="inlineStr">
+        <is>
+          <t>Observácia: sekcia 'Zadajte dopyt' + recenzia chváli filtrovanie vážnych záujemcov</t>
+        </is>
+      </c>
+      <c r="J309" s="10" t="inlineStr">
+        <is>
+          <t>Vysoká</t>
+        </is>
+      </c>
+      <c r="K309" s="10" t="inlineStr">
+        <is>
+          <t>Odoslané</t>
+        </is>
+      </c>
+      <c r="L309" s="10" t="inlineStr">
+        <is>
+          <t>16.07.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" s="10" t="n">
+        <v>349</v>
+      </c>
+      <c r="B310" s="10" t="inlineStr">
+        <is>
+          <t>Zdravotníctvo</t>
+        </is>
+      </c>
+      <c r="C310" s="10" t="inlineStr">
+        <is>
+          <t>Rehab Care s.r.o. (rehabilitačná klinika)</t>
+        </is>
+      </c>
+      <c r="D310" s="10" t="inlineStr">
+        <is>
+          <t>https://rehabcare.sk</t>
+        </is>
+      </c>
+      <c r="E310" s="10" t="inlineStr">
+        <is>
+          <t>[treba dohľadať]</t>
+        </is>
+      </c>
+      <c r="F310" s="10" t="inlineStr">
+        <is>
+          <t>+421 948 697 379</t>
+        </is>
+      </c>
+      <c r="G310" s="10" t="inlineStr">
+        <is>
+          <t>Košice</t>
+        </is>
+      </c>
+      <c r="H310" s="10" t="inlineStr">
+        <is>
+          <t>AI triage navigátor mapuje ťažkosť pacienta (napr. bolesť krížov) na správnu službu/terapeuta a rezervuje cez ich Bookio</t>
+        </is>
+      </c>
+      <c r="I310" s="10" t="inlineStr">
+        <is>
+          <t>Observácia: 30+ služieb, nový pacient nevie ktorá sedí na jeho problém</t>
+        </is>
+      </c>
+      <c r="J310" s="10" t="inlineStr">
+        <is>
+          <t>Vysoká</t>
+        </is>
+      </c>
+      <c r="K310" s="10" t="inlineStr">
+        <is>
+          <t>Treba lepší research</t>
+        </is>
+      </c>
+      <c r="L310" s="10" t="inlineStr">
+        <is>
+          <t>Súkromná fyzio klinika (nespolupracuje so ZP) + vzdelávacie centrum. Už majú Bookio online rezerváciu. Obrovský katalóg (SM systém, Vojtova, suchá ihla, ženská fyzio...). EMAIL NEZOBRAZENÝ NA HP - overiť na /kontakt. Silný hook na triage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="B311" s="10" t="inlineStr">
+        <is>
+          <t>Hotel/Penzión</t>
+        </is>
+      </c>
+      <c r="C311" s="10" t="inlineStr">
+        <is>
+          <t>Via Jasná – Apartmány</t>
+        </is>
+      </c>
+      <c r="D311" s="10" t="inlineStr">
+        <is>
+          <t>https://viajasna.sk</t>
+        </is>
+      </c>
+      <c r="E311" s="10" t="inlineStr">
+        <is>
+          <t>[treba dohľadať]</t>
+        </is>
+      </c>
+      <c r="F311" s="10" t="inlineStr">
+        <is>
+          <t>+421 904 318 042</t>
+        </is>
+      </c>
+      <c r="G311" s="10" t="inlineStr">
+        <is>
+          <t>Liptovský Mikuláš (Demänová)</t>
+        </is>
+      </c>
+      <c r="H311" s="10" t="inlineStr">
+        <is>
+          <t>AI asistent na web odpovie na opakované FAQ (wellness v cene?, psy?, check-in, kód LETO26) a dotiahne PRIAMU rezerváciu bez OTA provízií</t>
+        </is>
+      </c>
+      <c r="I311" s="10" t="inlineStr">
+        <is>
+          <t>Observácia: tlačia priamu rezerváciu + majú rozsiahle FAQ; 4,5/5 z 1812 recenzií</t>
+        </is>
+      </c>
+      <c r="J311" s="10" t="inlineStr">
+        <is>
+          <t>Vysoká</t>
+        </is>
+      </c>
+      <c r="K311" s="10" t="inlineStr">
+        <is>
+          <t>Treba lepší research</t>
+        </is>
+      </c>
+      <c r="L311" s="10" t="inlineStr">
+        <is>
+          <t>Apartmány+wellness+reštaurácia, 4,5/5 z 1812 Google recenzií. Aktívne tlačia priamu rezerváciu (zľava LETO26) proti OTA. Rozsiahle FAQ na webe = veľa opakovaných otázok. Recenzie chvália kuchyňu, drobné sťažnosti na upratovanie. EMAIL NEZOBRAZENÝ - overiť. Tón: rodinný, férové ceny.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:M31"/>

</xml_diff>